<commit_message>
Update existing files with accessibility improvements and benchmark results
</commit_message>
<xml_diff>
--- a/Combined_Benchmark_Results.xlsx
+++ b/Combined_Benchmark_Results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9d549c7b2720060c/Desktop/reportingxpress1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="228" documentId="8_{E92B2527-2DEA-40AF-B733-65139052A88F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{169B518F-0F4E-4978-ACF3-E04C12B6D0DA}"/>
+  <xr:revisionPtr revIDLastSave="248" documentId="8_{E92B2527-2DEA-40AF-B733-65139052A88F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5E6F6EE7-946B-4A08-A03D-827B98617E27}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{15A1E041-C4EC-4DA5-90DC-66ECF3AB2B49}"/>
+    <workbookView minimized="1" xWindow="3120" yWindow="3120" windowWidth="21600" windowHeight="11235" xr2:uid="{15A1E041-C4EC-4DA5-90DC-66ECF3AB2B49}"/>
   </bookViews>
   <sheets>
     <sheet name="Benchmark Summary" sheetId="10" r:id="rId1"/>
@@ -22,6 +22,7 @@
     <sheet name="Google Antigravity Update 2" sheetId="7" r:id="rId7"/>
     <sheet name="Google Antigravity Update 3" sheetId="8" r:id="rId8"/>
     <sheet name="Google Antigravity Update 4" sheetId="12" r:id="rId9"/>
+    <sheet name="Google Antigravity Update 5" sheetId="13" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1586" uniqueCount="1063">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1785" uniqueCount="1190">
   <si>
     <t>Timestamp</t>
   </si>
@@ -6411,6 +6412,767 @@
 4. **Tenure &amp; Lifetime Value (LTV) Analysis**: Understanding the tenure and lifetime value of your $1 million donors can reveal how long they typically remain engaged with your organization and the total value they bring over their lifetime. This analysis can help you refine your strategies for retaining and upgrading these donors [QX165].
 5. **Year-Over-Year Variance**: Reviewing the year-over-year variance in giving from your top donors can highlight trends and shifts in their giving behavior. This can inform your future fundraising strategies and help you identify any necessary adjustments in your approach to major gifts [QX44].
 By focusing on these analytics, you can gain a comprehensive understanding of your $1 million lifetime donors, their giving patterns, and the effectiveness of your engagement strategies. Blend these RFM-based analytics with engagement analytics for a better picture.</t>
+  </si>
+  <si>
+    <t>[QX146] | [QX88] | [QX47]</t>
+  </si>
+  <si>
+    <t>To identify top segment donors that are at risk of lapsing, you should focus on specific RFM (Recency, Frequency, Monetary Value) analytics that can provide insights into donor behavior and engagement patterns. Here are the key analytics you should consider:
+1. **Recently Lapsed Top Donors (15 months)**: This analysis will help you identify donors who have recently lapsed and are significant contributors. By examining their giving history, you can understand patterns that led to their lapse and strategize on how to re-engage them effectively [QX146].
+2. **Current Donors Major Gift Prospect Analysis**: This report focuses on your current major gift donors and includes metrics on outright lapse mitigation year-over-year. It can help you identify which major donors are showing signs of disengagement and may be at risk of lapsing [QX88].
+3. **Occasional Donor Analysis**: This analysis looks at donors who have given in 3 out of the last 5 years. Understanding this group can provide insights into those who may be on the verge of lapsing, allowing you to take proactive measures to retain them [QX47].
+4. **Recency and Frequency Metrics**: By analyzing the recency of donations (how recently a donor has given) and the frequency of their donations, you can pinpoint donors who have not engaged recently or have reduced their giving frequency. This can be a strong indicator of potential lapsing.
+5. **Monetary Value Trends**: Reviewing the monetary value of donations over time can help you identify donors whose contributions have significantly decreased. A drop in giving amount can signal a risk of lapsing, prompting you to reach out before they fully disengage.
+By blending these RFM-based analytics with engagement analytics, you can gain a more comprehensive view of your donors' behaviors and motivations, allowing for targeted re-engagement strategies. This approach will help you mitigate lapses and strengthen donor relationships.</t>
+  </si>
+  <si>
+    <t>[QX174] | [QX147] | [QX107] | CI Hub Modified FINAL LARGE DOC (1) (Page 27) | PreventDonorAttrition (1) (Page 2) | seasonal giving patterns (Page 2)</t>
+  </si>
+  <si>
+    <t>Before launching a campaign, it's crucial to review several key metrics that will provide insights into your donor base and help you make informed decisions. Here are the specific analytics you should focus on:
+1. **Retention Rate of New Donors**: Understanding how many of your new donors are retained after their first gift is essential. This metric will help you gauge the effectiveness of your onboarding and engagement strategies. A high retention rate indicates that your initial outreach is successful, while a low rate may signal the need for improved engagement tactics [QX174].
+2. **Average Gift Size**: Monitoring the increase in average gift size over time can provide insights into donor behavior and the effectiveness of your fundraising strategies. If you notice a trend of increasing average gifts, it may suggest that your messaging and engagement efforts are resonating with your supporters [QX107].
+3. **Conversion Rate of New Donors to Recurring Donors**: This metric tracks how effectively you are converting one-time donors into recurring supporters. A higher conversion rate indicates successful engagement and retention strategies, which are critical for long-term fundraising success [QX174].
+4. **Lapsed Donor Re-engagement Metrics**: If you have previously lapsed donors, tracking the percentage of these donors who re-engage and make new gifts following targeted outreach is vital. This will help you assess the effectiveness of your re-engagement campaigns and refine your strategies accordingly [QX147].
+5. **Incremental Lift Analysis**: Review the incremental lift in donations during specific periods, especially after implementing targeted campaigns. This analysis can help you understand the impact of your outreach efforts and set realistic performance benchmarks for future campaigns [QX107].
+By focusing on these metrics, you can gain a comprehensive understanding of your donor landscape and make data-driven decisions that enhance your campaign's effectiveness. Remember, blending these RFM-based analytics with engagement analytics will provide a better picture of your donor relationships and campaign potential.</t>
+  </si>
+  <si>
+    <t>[QX71] | Nyman Pilbeam Baines Maklan 2016 Transformational Gifts Roles Accepted Manuscript (Page 27) | Shaker 2018 Understanding Higher Education Fundraisers Report (Page 6) | Shaker Nelson 2021 Grounded Theory Major Gift Relationships (Page 11) | Karlan List 2006 Does Price Matter in Charitable Giving NBER W12338 (Page 5) | Stanford PACS 2020 Community Based Orgs High Capacity Donors (Page 33)</t>
+  </si>
+  <si>
+    <t>To understand the roles of fundraisers in securing transformational gifts, you can focus on several key activities that are essential for building relationships and facilitating significant donations. Here are the primary roles and their associated activities:
+1. **Networker**: Fundraisers must build personal, trusted relationships with donors, their families, and other advisors. This involves developing strong connections with organizational leaders to foster a supportive environment for giving [Nyman Pilbeam Baines Maklan 2016, Page 27].
+2. **Negotiator**: This role requires fundraisers to create a change-ready organization and establish visionary goals. They must maintain a long-term funding perspective and understand the donor's intentions, ensuring that the impact of donations is clearly communicated [Nyman Pilbeam Baines Maklan 2016, Page 27].
+3. **Knowledge Broker**: Fundraisers need to possess knowledge of wealth management strategies, including tax laws, and monitor the wealth of current clients. This knowledge helps them refresh their pool of potential donors and tailor their approaches accordingly [Nyman Pilbeam Baines Maklan 2016, Page 27].
+4. **Personalized Association Builder**: Fundraisers should form personalized associations with donors by planning tailored interactions. This involves gathering insights about donors' personalities, preferences, and priorities, which can be used to create strategic action plans for engagement [Shaker Nelson 2021, Page 11].
+5. **Strategic Solicitor**: Fundraisers must be able to distill information and strategically solicit prospective donors. This requires behavioral and linguistic flexibility, intellectual curiosity, and the ability to understand both the institution's needs and the donor's motivations [Shaker 2018, Page 6].
+By focusing on these roles and activities, fundraisers can enhance their effectiveness in securing transformational gifts, ultimately leading to deeper donor relationships and increased philanthropic support for their organizations.
+For a more comprehensive understanding, consider blending these insights with RFM analytics, such as donor retention rates and the growth of active donor counts, to assess the effectiveness of your fundraising strategies over time [QX71].</t>
+  </si>
+  <si>
+    <t>[QX159] | [QX158] | [QX167] | CI Hub Modified FINAL LARGE DOC (1) (Page 39)</t>
+  </si>
+  <si>
+    <t>To improve major donor retention, you should focus on several key RFM-based analytics that can provide insights into donor behavior and potential upgrade opportunities. Here are the specific analytics you should consider:
+1. **Top Segment Stable-Target Increase**: This analytic identifies upgrade candidates from your top-segment donor pool. By examining donors who have consistently given at a stable level over the past two years, you can pinpoint those who may be ready to increase their contributions. This analysis utilizes historical giving data to assess contribution patterns, which can help you tailor your engagement strategies to encourage higher giving levels [QX159].
+2. **Bottom Segment Stable-Target Increase**: While focusing on major donors, itâ€™s also beneficial to look at the bottom segment. This analysis identifies potential upgrade candidates from donors who have shown stable giving patterns. Understanding these donors can help you develop strategies to elevate them into higher giving tiers, which can ultimately contribute to overall retention efforts [QX158].
+3. **Bottom Segment Donor Loyalty Analysis**: This analytic provides insights into donor loyalty specifically among your bottom segment. By tracking giving patterns and identifying trends, you can develop targeted strategies aimed at retaining these donors. Key metrics include the current streak of consecutive years a donor has contributed and any upward movement into higher tiers, which can signal potential for increased engagement and giving [QX167].
+4. **Donor Retention Patterns**: Research indicates that retaining donors is significantly less expensive than acquiring new ones, and recurring donors typically give more than one-time donors. Understanding the retention patterns across different donor segments can help you tailor your stewardship approaches effectively [CI Hub Modified FINAL LARGE DOC (1) (Page 39)].
+5. **Segmentation Analysis**: Conducting a segmentation analysis can reveal how different donor groups behave and their likelihood of retention. This can help you identify which segments require different stewardship approaches, allowing you to allocate resources more effectively and improve retention rates [CI Hub Modified FINAL LARGE DOC (1) (Page 39)].
+By leveraging these RFM-based analytics, you can gain a clearer understanding of your major donors' behaviors and preferences, which will inform your strategies for improving retention. Remember to blend these RFM-based analytics with engagement analytics for a better picture of your donor relationships.</t>
+  </si>
+  <si>
+    <t>[QX146] | [QX69] | [QX65] | CI Hub Modified FINAL LARGE DOC (1) (Page 26)</t>
+  </si>
+  <si>
+    <t>To effectively handle a donor who has stopped giving, you should focus on analyzing specific RFM metrics that can provide insights into their past behavior and potential for re-engagement. Here are the key analytics you should consider:
+1. **Recent Top Donor Recaptures Analysis**: This analysis will help you identify donors who have previously lapsed and successfully returned. It provides a historical log of recapture events, detailing the duration of their lapse, previous giving levels, and total contributions. Understanding these patterns can inform your reactivation strategies and help you tailor your outreach efforts effectively [QX65].
+2. **Lapse Prevention Toolkit**: Utilize this toolkit to monitor the total value of contributions from re-engaged donors and track improvements in donor retention rates over time. This will allow you to evaluate the effectiveness of your re-engagement strategies and adjust them as necessary [QX146].
+3. **Months Lapsed Metric**: This metric can be particularly useful in testing new timing for reactivation campaigns. By analyzing how long donors have been lapsed, you can craft personalized messaging that acknowledges their previous commitment and encourages them to return [QX69].
+4. **Retention Hub**: Review your organization's retention rates and identify any warning signs, such as a retention cliff or accelerating lapse rates. This will help you understand if there are systemic issues in your engagement strategies that need to be addressed [CI Hub Modified FINAL LARGE DOC (1) (Page 26)].
+5. **Strategic Reactivation Success Rates**: Look at sector benchmarks for reactivation rates, which suggest that donors lapsed for less than two years have a reactivation success rate of 8-12%. This can guide your expectations and strategies for reaching out to lapsed donors [CI Hub Modified FINAL LARGE DOC (1) (Page 26)].
+By focusing on these RFM-based analytics, you can develop a targeted approach to re-engage lapsed donors. Remember to blend these RFM-based analytics with engagement analytics for a better picture of your donor's behavior and preferences.</t>
+  </si>
+  <si>
+    <t>[QX57] | [QX63] | [QX12] | CI Hub Modified FINAL LARGE DOC (1) (Page 24) | PreventDonorAttrition (1) (Page 2) | seasonal giving patterns (Page 2)</t>
+  </si>
+  <si>
+    <t>To assess how your organization is performing this year compared to last year, you should focus on several key RFM-based analytics that will provide insights into donor behavior and retention. Here are the specific metrics and analyses you should consider:
+1. **Overall Retention Rate**: This metric will help you understand the percentage of donors from last year who have given again this year. Itâ€™s crucial for evaluating donor loyalty and the effectiveness of your stewardship efforts [QX12].
+2. **First-Year Donor Retention**: Analyze how many new donors from last year have made a second gift this year. This is a critical indicator of your ability to convert first-time donors into repeat supporters [QX57].
+3. **Multi-Year Retention**: Look at the patterns of donors who have given in consecutive years (2+, 3+, 5+ years). This will help you identify trends in donor loyalty over time and assess whether your long-term retention strategies are effective [QX63].
+4. **Year-Over-Year Variance in Donor Counts and Gift Amounts**: Compare the total number of donors and the overall dollars raised this year against last year. This will provide a clear picture of growth or decline in your fundraising efforts [PreventDonorAttrition (1), Page 2].
+5. **Gift Behavior Analysis**: Examine how many of your retained donors have upgraded, downgraded, or maintained their giving levels compared to last year. This will help you understand the financial health of your donor base and identify areas for improvement [PreventDonorAttrition (1), Page 2].
+By reviewing these metrics, you can gain a comprehensive understanding of your organization's performance this year relative to last year. Remember, blending these RFM-based analytics with engagement analytics will provide a better picture of your overall fundraising effectiveness.</t>
+  </si>
+  <si>
+    <t>[QX167] | [QX161] | [QX77] | CI Hub Modified FINAL LARGE DOC (1) (Page 6)</t>
+  </si>
+  <si>
+    <t>To determine if your organization is on track to meet its annual fundraising goal, you should focus on several key RFM-based analytics that can provide insights into your donor behavior and revenue trends. Here are the specific analytics you should review:
+1. **Active Donor Loyalty Summary Analysis by Segment**: This analysis will help you track retention rates, average gift trends, and gift frequency across different donor segments (Top, Middle, Bottom). Understanding these metrics is crucial, as a decline in retention rates, especially among your Active Top Segment, can significantly impact your overall revenue [QX77].
+2. **Bottom Segment Donor Loyalty Analysis**: This analytic focuses on the loyalty of donors in the Bottom Segment. By examining their giving patterns, you can identify trends that may affect your annual goal. Key metrics include the total annual giving for each constituent and their historical giving streaks, which can indicate potential for increased engagement and giving [QX167].
+3. **Segment-Specific Year-Over-Year Metrics**: This review will allow you to monitor retention rates and average gift trends across all segments. Itâ€™s essential to understand how each segment is performing relative to your annual goal, as different segments contribute differently to your overall revenue [CI Hub Modified FINAL LARGE DOC (1) (Page 6)].
+4. **Outright Lapse Mitigation Year-Over-Year**: This analysis can help you identify any lapses in donor engagement and retention, which could hinder your progress toward your annual goal. By focusing on mitigating lapses, you can implement strategies to re-engage donors who may be at risk of dropping off [QX161].
+5. **Cohort Analysis for Retention**: Evaluating the retention rates at one, two, and five-year milestones can provide insights into how well you are maintaining donor relationships over time. This is critical for understanding if you are on track to meet your annual fundraising targets [QX161].
+By reviewing these analytics, you can gain a clearer picture of your current fundraising performance and identify areas that may need attention to ensure you meet your annual goal. Remember, blending these RFM-based analytics with engagement analytics will provide a better picture of your overall fundraising health.</t>
+  </si>
+  <si>
+    <t>[QX24] | [QX27] | [QX54] | seasonal giving patterns (Page 4) | PreventDonorAttrition (1) (Page 2) | CI Hub Modified FINAL LARGE DOC (1) (Page 4)</t>
+  </si>
+  <si>
+    <t>To understand the change in your revenue from last year, you should focus on several key RFM (Recency, Frequency, Monetary Value) analytics that can provide insights into donor behavior and financial performance. Here are the specific analytics you should review:
+1. **Overall Donor Counts and Retention Rates**: Analyze the total number of donors and the retention rates over the past year. This will help you identify if changes in donor retention have significantly impacted your revenue. Pay particular attention to retention rates sliced by consecutive years of giving, especially for those in their second year, as this is a critical retention milestone [PreventDonorAttrition (1), Page 2].
+2. **Average Gift Size and Total Transaction Volume**: Review the average gift size and the total number of gifts received. This will help you determine whether revenue changes are due to an increase in the number of transactions or changes in the average gift size. Understanding whether growth comes from donor upgrading or simply more transactions is crucial [CI Hub Modified FINAL LARGE DOC (1), Page 4].
+3. **Frequency Changers Analysis**: Look at the "frequency changers" metric, which indicates how many donors adjusted their giving cadence. This analysis can reveal shifts in donor behavior that may have influenced revenue, such as an increase in donors giving more frequently or a decrease in those who have lapsed [QX24].
+4. **Seasonal Giving Patterns**: Examine seasonal giving patterns to see if there were specific months or quarters where revenue increased or decreased. This can provide insights into the effectiveness of your campaigns and whether they aligned with donor behavior [Seasonal Giving Patterns (Page 4)].
+5. **Donor Lifecycle Analysis**: Assess the donor lifecycle to understand the share of donors retained, renewed, or acquired each year. This will help you identify if a shrinking share of retained donors is contributing to revenue changes, indicating a potential "leaky bucket" scenario [CI Hub Modified FINAL LARGE DOC (1), Page 4].
+By analyzing these RFM-based metrics, you can gain a clearer picture of the factors driving changes in your revenue. Remember to blend these RFM-based analytics with engagement analytics for a better picture, as engagement data can provide additional context on donor interactions and campaign effectiveness.</t>
+  </si>
+  <si>
+    <t>[QX27] | [QX57] | [QX74] | seasonal giving patterns (Page 4) | CI Hub Modified FINAL LARGE DOC (1) (Page 39)</t>
+  </si>
+  <si>
+    <t>To analyze your organization's giving history over many years, you should focus on several key RFM-based analytics that will provide insights into donor behavior and trends. Here are the specific analytics you should review:
+1. **Lifetime Giving Analysis**: This metric will help you understand the total contributions made by donors over their lifetime. It allows you to identify which donor cohorts have the highest lifetime value and how their giving patterns have evolved over time. This analysis is crucial for forecasting future revenue and refining your stewardship strategies [QX27].
+2. **Tenure Analysis**: Reviewing the average tenure of your donors will give you insights into how long donors typically stay engaged with your organization. This metric can help you identify patterns in donor retention and understand which cohorts are most likely to continue giving [QX27].
+3. **Cohort Analysis**: By grouping donors based on their fiscal year of acquisition, you can track how different cohorts perform over time. This analysis will reveal which acquisition strategies have been most effective and help you pinpoint areas for improvement in donor retention and upgrades [QX57].
+4. **Anniversary Retention Rates**: This metric measures the percentage of donors who give again in the same month they were acquired. It is particularly useful for assessing the effectiveness of your onboarding and stewardship efforts for new donors. Understanding these rates can guide your engagement strategies and help you optimize follow-up efforts [QX74].
+5. **Seasonal Giving Patterns**: Analyzing seasonal trends in giving can provide insights into when donors are most likely to contribute. This information can be leveraged to time your campaigns effectively and align your stewardship efforts with natural donor behavior patterns [Seasonal Giving Patterns (Page 4)].
+By reviewing these analytics, you will gain a comprehensive understanding of your giving history and be better equipped to refine your fundraising strategies. Remember to blend these RFM-based analytics with engagement analytics for a better picture of donor behavior and engagement.</t>
+  </si>
+  <si>
+    <t>[QX139] | [QX54] | [QX180] | PreventDonorAttrition (1) (Page 2) | seasonal giving patterns (Page 4) | CI Hub Modified FINAL LARGE DOC (1) (Page 18)</t>
+  </si>
+  <si>
+    <t>To gain insights into what your revenue might look like next year, you should focus on several key RFM-based analytics that can help you model future performance. Here are the specific analytics you should consider:
+1. **Projected Donor Count and Projected Revenue Analysis**: This analysis will help you understand potential shifts in donor segments and quantify your future pipeline. By examining projected counts and revenue for different giving levels, you can set realistic targets and identify areas that may require more attention, such as high-touch engagement for at-risk donors [QX139].
+2. **Donor Lifecycle Analysis**: This involves examining the share of donors retained, renewed, or acquired each year. Understanding the trends in donor behavior, including upgrades and downgrades, will provide a clearer picture of your revenue flow and help you identify potential areas for growth or improvement [PreventDonorAttrition (1) (Page 2)].
+3. **Retention Patterns**: Analyzing retention rates, especially for donors in their second year, is crucial. This metric can reveal how well you are maintaining your donor base and can indicate future revenue stability. Pay attention to retention rates sliced by gift band, particularly for those giving at or above your organizationâ€™s median gift size [PreventDonorAttrition (1) (Page 2)].
+4. **Seasonal Giving Patterns**: Understanding seasonal trends in donor behavior can inform your revenue projections. By analyzing when donors are most likely to give, you can align your fundraising campaigns with these patterns, potentially increasing your revenue during peak times [seasonal giving patterns (Page 4)].
+5. **Revenue Gains and Losses by Donor Category**: This analysis categorizes donors into groups such as New, Lapsed, Increased, Decreased, and Same. By understanding where your revenue is coming from and where it is being lost, you can develop targeted strategies to retain and re-engage donors, which is essential for forecasting future revenue [QX180].
+By integrating these RFM-based analytics, you can create a more informed projection of your revenue for the upcoming year. However, to enhance your understanding, consider blending these RFM-based analytics with engagement analytics for a better picture. This will provide a more comprehensive view of donor behavior and potential revenue outcomes.</t>
+  </si>
+  <si>
+    <t>[QX40] | [QX141] | [QX159] | CI Hub Modified FINAL LARGE DOC (1) (Page 14)</t>
+  </si>
+  <si>
+    <t>To assess how dependent your organization is on your top donors, you should focus on several key RFM-based analytics that will provide insights into donor concentration and revenue reliance. Here are the specific analytics you should consider:
+1. **Concentration Ratio Analysis**: This analysis will help you understand the percentage of total revenue that comes from your top donor segments. By tracking changes in the concentration ratio over time, you can evaluate whether your organization is becoming overly reliant on a small group of donors or if you are successfully broadening your donor base [QX40].
+2. **Top Segment Stable-Target Increase**: This analytic identifies upgrade candidates within your top-segment donor pool. By examining donors who have consistently given at a stable level over the past two years, you can determine if these donors are likely to continue their support or if they represent a risk of becoming less engaged. This will help you gauge the stability of your top donor contributions [QX159].
+3. **Donor Segmentation Analysis**: Segmenting your donors into categories (Top, Middle, Bottom) allows you to see how many donors are contributing to your overall revenue. This analysis can highlight whether your revenue is concentrated among a few top donors or if you have a more diverse donor base [QX141].
+4. **Trend Analysis of Donor Contributions**: By reviewing historical giving data, you can identify trends in donor contributions over time. This will help you understand if your top donors are increasing their contributions, maintaining them, or if there are signs of potential lapses [QX159].
+5. **Emerging Concentration Risk Assessment**: This assessment can illustrate the potential risks associated with donor concentration. For example, if a small percentage of your donors contribute a large portion of your revenue, it indicates a high concentration risk. Understanding this can inform your strategies to diversify your donor base [CI Hub Modified FINAL LARGE DOC (1), Page 14].
+By focusing on these analytics, you can gain a clearer picture of your dependency on top donors and develop strategies to mitigate risks associated with donor concentration. Remember, blending these RFM-based analytics with engagement analytics will provide a better picture of your donor landscape.</t>
+  </si>
+  <si>
+    <t>[QX167] | [QX40] | [QX166] | CI Hub Modified FINAL LARGE DOC (1) (Page 39)</t>
+  </si>
+  <si>
+    <t>To understand your giving pyramid, you should focus on the **Top 50% Donor Concentration Analysis**. This analysis will provide insights into how much of your total donations come from your top donor segments, specifically examining the cumulative giving of the top 5%, 10%, 15%, up to 50% of your donor base over the current and prior fiscal years. By analyzing this data, you can determine the proportion of your total fundraising that is reliant on your highest-contributing supporters, which is crucial for understanding the overall health of your fundraising strategy [QX40].
+Additionally, consider the **Bottom Segment Donor Loyalty Analysis** and the **Middle Segment Donor Loyalty Analysis**. These analyses will help you understand the loyalty and giving patterns of donors in the lower and middle tiers of your pyramid. The Bottom Segment analysis focuses on identifying trends in donor behavior and retention among your least engaged donors, while the Middle Segment analysis examines the consistency of support from mid-level donors and their potential for upgrading to higher tiers [QX167][QX166].
+By combining insights from these three analyses, you can gain a comprehensive view of your giving pyramid, including where your revenue is concentrated and how different segments are performing. This understanding will enable you to develop targeted strategies for donor engagement and retention across all levels of your donor base.
+Blend these RFM-based analytics with engagement analytics for a better picture.</t>
+  </si>
+  <si>
+    <t>[QX153] | [QX155] | [QX99] | Stanford PACS 2020 Community Based Orgs High Capacity Donors (Page 21) | Stanford PACS 2020 How We Give Now Report (Page 60) | CI Hub Modified FINAL LARGE DOC (1) (Page 21)</t>
+  </si>
+  <si>
+    <t>To identify who made the largest gifts last year, you should focus on the following analytics:
+1. **Top Donors whose gift size is Increasing**: This analytic will help you identify donors who were in the 'Top' giving segment during the last full fiscal year and whose average gift size has increased compared to the previous year. By analyzing their total and average gift amounts over the last three fiscal years, you can pinpoint significant contributors and understand their giving behavior [QX153].
+2. **Largest Gifts Analysis**: This analysis provides insights into each donor's total giving last year, the amount and date of their largest gift, and a percentile indicator showing how their top gift compares to the middle segment. This will allow you to quickly identify major donors and personalize your outreach based on their previous engagement [QX99].
+3. **Gift Size and Seasonality**: Understanding the composition of your gifts can reveal whether your largest gifts come from a few major donors or a broader base of smaller contributions. This analysis can help you assess the risk of revenue vulnerability due to individual donor attrition and identify opportunities for upgrade campaigns [CI Hub Modified FINAL LARGE DOC (1), Page 21].
+4. **Bottom Donors whose gift size is Increasing**: While this analytic focuses on donors in the 'Bottom' giving segment, it can still provide valuable insights into those who are increasing their average gift size. This may help you identify potential future major donors who are on the rise [QX155].
+By reviewing these analytics, you will gain a comprehensive understanding of your largest donors and their giving patterns. Remember to blend these RFM-based analytics with engagement analytics for a better picture.</t>
+  </si>
+  <si>
+    <t>[QX145] | [QX19] | [QX82] | Stanford PACS 2020 How We Give Now Report (Page 37) | Stanford PACS 2018 Data for Donor Impact (Page 16) | Stanford PACS 2020 Community Based Orgs High Capacity Donors (Page 23)</t>
+  </si>
+  <si>
+    <t>To analyze the split between individual and organizational giving, you should focus on the following RFM-based analytics:
+1. **Top Segment Analysis**: This will help you identify your most valuable supporters by segmenting your donors into individuals and organizations. Understanding the trends in giving from these two groups will provide insights into how well you are engaging with each segment and inform your outreach strategies [QX145].
+2. **Organizational Giving Assessment**: This analysis will allow you to evaluate how much funding is coming from corporate partners versus individual donors. By assessing the trends in individual versus organizational giving, you can tailor your fundraising strategies accordingly. For instance, if individual giving is declining, you might need to implement strategies to re-engage those donors [QX145].
+3. **Giving Trend Analysis**: This involves tracking the changes in giving over time, categorized by significant increases, modest increases, or decreases. This will help you understand the dynamics of both individual and organizational contributions and identify any shifts in donor behavior [QX19].
+4. **Performance Score Review**: This analysis distills complex giving trajectories into a concise signal for each donor, helping you identify who is increasing their giving, who has lapsed, and who has been newly reactivated. This can provide context for understanding the overall health of both individual and organizational giving [QX82].
+5. **Annual Review of Giving Trends**: Conducting an annual review at the close of the fiscal year will align your findings with your reporting and strategy planning cycles. This will help you assess the overall split between individual and organizational giving and make informed decisions for future fundraising efforts [QX145].
+By focusing on these RFM-based analytics, you can gain a clearer picture of the split between individual and organizational giving. Blend these RFM-based analytics with engagement analytics for a better picture.</t>
+  </si>
+  <si>
+    <t>[QX57] | [QX51] | [QX178] | CI Hub Modified FINAL LARGE DOC (1) (Page 24) | Stanford PACS 2020 How We Give Now Report (Page 60) | PreventDonorAttrition (1) (Page 2)</t>
+  </si>
+  <si>
+    <t>To assess your donor retention rate, you should focus on several key RFM-based analytics that will provide insights into your donor behavior over time. Here are the specific metrics you should review:
+1. **Overall Retention Rate**: This metric tracks the percentage of donors from the previous year who made a contribution again in the current year. It gives you a clear picture of how well you are retaining your existing donor base [QX178].
+2. **First-Year Donor Retention**: This metric measures the conversion of new donors to their second gift. It's crucial to understand how effectively you are engaging new donors early in their relationship with your organization [QX51].
+3. **Multi-Year Retention**: Analyze the patterns of donors who have given in consecutive years (2+, 3+, 5+ year patterns). This will help you identify long-term loyalty trends among your donor base [QX178].
+4. **Retention Rates by Acquisition Year**: This analysis allows you to see how many donors from specific acquisition years are retained, which can highlight the effectiveness of your onboarding and stewardship strategies [QX51].
+5. **Donor Lifecycle Analysis**: Understanding the share of your donors who were retained, renewed, or newly acquired each year can provide insights into your overall donor health and retention strategies [PreventDonorAttrition].
+By reviewing these metrics, you can gain a comprehensive understanding of your donor retention rates and identify areas for improvement. Remember, blending these RFM-based analytics with engagement analytics will provide a better picture of your donor relationships and retention strategies.</t>
+  </si>
+  <si>
+    <t>[QX15] | [QX159] | [QX91] | CI Hub Modified FINAL LARGE DOC (1) (Page 37)</t>
+  </si>
+  <si>
+    <t>To assess the loyalty of your top donors, you should focus on several key RFM-based analytics that will provide insights into their giving behavior and retention patterns. Here are the specific analyses you should consider:
+1. **Second to Third Gift Retention Analysis**: This analysis is crucial for understanding how effectively you retain donors between their second and third gifts. It examines the journey of donors who have made at least two contributions, allowing you to see the percentage of these donors who make a third gift. Additionally, it provides insights into how quickly they progress from their first to second and second to third gifts, which is vital for gauging loyalty [QX15].
+2. **Top Segment Stable-Target Increase**: This analytic identifies potential upgrade candidates within your top-segment donor pool by examining those who have consistently given at a stable level over the past two years. By focusing on donors who have maintained or increased their contributions, you can identify loyal supporters who may be ready for an upgrade, thus reflecting their ongoing commitment to your organization [QX159].
+3. **Gift Size Distribution + Donor Retention Cohort Analysis**: This combination analysis reveals how giving patterns correlate with retention behavior across different donor segments. By understanding which gift sizes correlate with higher retention rates, you can better assess the loyalty of your top donors and tailor your engagement strategies accordingly [CI Hub Modified FINAL LARGE DOC (1) (Page 37)].
+4. **Bottom Segment Gift Amount Trends**: While this analysis primarily focuses on lower-tier donors, it can provide context for understanding the overall giving landscape. By examining trends in gift amounts, you can identify if there are any concerning patterns among your top donors that might indicate a decline in loyalty [QX91].
+By utilizing these RFM-based analytics, you can gain a comprehensive view of your top donors' loyalty. However, to enhance your understanding, consider blending these RFM-based analytics with engagement analytics for a better picture. This will allow you to see how engagement efforts may influence donor loyalty and retention.</t>
+  </si>
+  <si>
+    <t>[QX163] | [QX167] | [QX170] | CI Hub Modified FINAL LARGE DOC (1) (Page 6)</t>
+  </si>
+  <si>
+    <t>To identify donors who give occasionally but not consistently, you should focus on the following RFM-based analytics:
+1. **Bottom Segment Donor Loyalty Analysis**: This analysis specifically examines the giving patterns of donors categorized in the Bottom Segment. It tracks their total annual giving, the streak of consecutive years they have contributed, and their historical maximum streak length. By understanding these metrics, you can identify donors who may give sporadically and assess their potential for increased engagement and retention [QX167].
+2. **Small-Dollar Segment Analysis**: Review the Small-Dollar Segment Analysis, which focuses on participation trends and retention rates. This segment often includes donors who give occasionally. By monitoring these metrics, you can identify patterns in giving frequency and determine which donors are not consistently contributing [CI Hub Modified FINAL LARGE DOC (1) (Page 6)].
+3. **Active Middle Segment Analysis**: This analysis can help you monitor upgrade patterns and retention rates among donors who may be giving occasionally. Since the middle segment often represents a potential upgrade pipeline, understanding their giving behavior can provide insights into those who are not consistently engaged [CI Hub Modified FINAL LARGE DOC (1) (Page 6)].
+4. **Consecutive Donors Analysis**: This analytic allows you to view the average and median annual giving of donors in each segment, including those who may not be consistently giving. By comparing these metrics, you can identify donors who have given in the past but may not have contributed recently, helping you to prioritize outreach efforts [QX170].
+By leveraging these RFM-based analytics, you can gain a clearer picture of your occasional donors. However, to enhance your understanding, consider blending these RFM-based analytics with engagement analytics for a better picture. This will allow you to assess the effectiveness of your outreach strategies and tailor your engagement efforts accordingly.</t>
+  </si>
+  <si>
+    <t>[QX161] | [QX46] | [QX74] | CI Hub Modified FINAL LARGE DOC (1) (Page 38)</t>
+  </si>
+  <si>
+    <t>To understand how long your donors typically stay active, you should focus on the following analytics:
+1. **Donor Tenure Distribution by Initial Segment**: This analytic will provide insights into how long donors remain active based on the segment they were in during their first year of giving (Top, Middle, Bottom). It includes average and median tenure in years for each segment, as well as the percentage of active years relative to their total tenure. This will help you gauge donor engagement over time and retention effectiveness across different segments [QX161].
+2. **3-Year Consecutive Donor Retention**: This analysis will allow you to see the retention rates of donors over a three-year period. It can help you identify trends in donor retention and understand how many donors continue to give year after year, which is crucial for assessing long-term donor relationships [QX46].
+3. **First Time Donors by Month and Retention**: This analytic will help you track the retention of first-time donors over time. Understanding how many of these new donors continue to give after their initial contribution can provide valuable insights into your organization's ability to convert first-time donors into long-term supporters [QX74].
+4. **Tenure &amp; Lifetime Value (LTV) by Segment**: This analysis combines donor tenure with their lifetime value, offering a comprehensive view of the economic impact of your donor relationships. It can help you identify which segments of donors are most valuable over time and how long they typically stay active, which is essential for strategic resource allocation [CI Hub Modified FINAL LARGE DOC (1) (Page 38)].
+By examining these analytics, you will gain a clearer picture of donor activity duration and retention trends within your organization. Remember, blending these RFM-based analytics with engagement analytics will provide a better overall understanding of donor behavior and retention strategies.</t>
+  </si>
+  <si>
+    <t>[QX91] | [QX163] | [QX161] | CI Hub Modified FINAL LARGE DOC (1) (Page 26)</t>
+  </si>
+  <si>
+    <t>To understand how donors move between segments over time, you should focus on the following analytics and metrics:
+1. **Segment Migration Analysis**: This analysis will help you track how donors transition between different segments (Top, Middle, Bottom) over specified timeframes. By examining the movement of donors, you can identify patterns and trends in donor behavior, which can inform your retention strategies and targeted outreach efforts [QX163].
+2. **Retention Hub**: This metric will provide insights into the retention rates of each donor segment. By analyzing the retention rates over time, you can determine how effectively you are maintaining relationships with different segments and identify any significant drops in retention that may require further investigation [QX161].
+3. **Gift Amount Trends (Annual)**: Reviewing the annual gift amounts by segment can reveal how donor contributions change over time. This analysis can help you understand if donors are upgrading to higher giving tiers or if there are trends indicating a decline in giving within certain segments [QX91].
+4. **Cohort Analysis**: This approach allows you to evaluate the behavior of specific groups of donors who joined during the same time period. By comparing the performance of these cohorts over time, you can gain insights into how different segments evolve and how your engagement strategies impact their giving behavior [QX163].
+5. **Donor Lifecycle Data**: Utilize your CI Hub Donor Lifecycle analytics to interpret your organization's actual rates of donor movement between segments. This data will provide a clearer picture of how your donor base is changing and help you benchmark against sector performance ranges [CI Hub Modified FINAL LARGE DOC (1) (Page 26)].
+By focusing on these analytics, you can gain a comprehensive understanding of donor movement between segments and make informed decisions to enhance your fundraising strategies. Remember to blend these RFM-based analytics with engagement analytics for a better picture.</t>
+  </si>
+  <si>
+    <t>[QX162] | [QX47] | [QX69] | CI Hub Modified FINAL LARGE DOC (1) (Page 54)</t>
+  </si>
+  <si>
+    <t>To identify which donors are about to lapse, you should focus on several key RFM-based analytics that can provide insights into donor behavior and predict potential lapses. Here are the specific analytics you should review:
+1. **Recency Analysis**: This metric will help you understand how recently donors have made contributions. Donors who have not given in a while are at a higher risk of lapsing. By analyzing the recency of donations, you can identify those who may need immediate attention to prevent them from lapsing [QX162].
+2. **Frequency Analysis**: Look at how often donors have contributed over a specific period. A decline in the frequency of donations can indicate that a donor is becoming disengaged. This analysis can help you pinpoint donors who may be on the verge of lapsing due to reduced giving activity [QX47].
+3. **Lapsing Donor Recovery Probability Analysis**: This predictive scoring system focuses on donors who have lapsed within the last 12 to 24 months. It identifies which of these donors are most likely to be successfully reactivated based on their historical giving patterns. This analysis can help you prioritize your outreach efforts effectively [CI Hub Modified FINAL LARGE DOC (1), Page 54].
+4. **Outright Lapse Mitigation YOY**: Reviewing this analysis can provide insights into trends in donor lapses over the years. It can help you understand which segments are most likely to lapse and the effectiveness of your past outreach efforts, allowing you to tailor your reactivation strategies accordingly [QX69].
+5. **Occasional Donor Analysis**: This analysis focuses on donors who give occasionally (3 out of 5 years). Understanding the patterns of these donors can help you identify those who are at risk of lapsing and develop targeted strategies to engage them before they stop giving altogether [QX47].
+By leveraging these RFM-based analytics, you can gain a clearer picture of which donors are at risk of lapsing and take proactive steps to engage them. **Blend these RFM-based analytics with engagement analytics for a better picture** to enhance your outreach efforts and improve donor retention.</t>
+  </si>
+  <si>
+    <t>[QX146] | [QX65] | [QX69]</t>
+  </si>
+  <si>
+    <t>To identify which top donors have already lapsed, you should focus on several key RFM-based analytics that will provide insights into donor behavior and engagement history. Here are the specific analytics you should consider:
+1. **Lapse Prevention Toolkit**: This toolkit will help you analyze recently lapsed top donors, focusing on their giving patterns before they lapsed. By examining the recency of their last donation, you can identify those who have not contributed recently and may need targeted re-engagement efforts [QX146].
+2. **Donor Recapture Analysis**: Look into the metrics surrounding the months lapsed between gifts and the giving levels before and after lapse. This analysis will help you understand how many top donors have lapsed and the potential for their return based on their historical giving behavior [QX65].
+3. **Recapture Rates**: Assess the recapture rates of lapsed donors, which will provide insights into how effectively you have been able to re-engage these individuals. This metric can also highlight trends in donor lapses and the effectiveness of your outreach strategies [QX69].
+4. **Giving Level Changes**: Evaluate the changes in giving levels of lapsed donors upon recapture. This will help you identify not only who has lapsed but also how their giving patterns have evolved, which can inform your future engagement strategies [QX65].
+5. **Segmentation of Donor Behavior**: Utilize segmentation to categorize lapsed donors based on their previous giving levels and engagement history. This will allow you to prioritize outreach to those who are most likely to return to or exceed their previous giving levels [QX69].
+By focusing on these RFM-based analytics, you can effectively identify and strategize around your lapsed top donors. Remember, blending these RFM-based analytics with engagement analytics will provide a more comprehensive picture of your donor landscape and enhance your re-engagement efforts.</t>
+  </si>
+  <si>
+    <t>[QX154] | [QX156] | [QX91] | CI Hub Modified FINAL LARGE DOC (1) (Page 25)</t>
+  </si>
+  <si>
+    <t>To identify donors who are giving less than they used to, you should focus on the following analytics:
+1. **Top Donors whose Gift Size is Decreasing**: This analytic will help you pinpoint donors who were classified as 'Top' givers in the last fiscal year but have shown a decrease in their average gift size compared to the previous year. By analyzing their giving patterns over the last three fiscal years, you can identify those at risk of disengagement and target them for renewed engagement efforts [QX154].
+2. **Bottom Donors whose Gift Size is Decreasing**: This analysis focuses on donors in the 'Bottom' giving segment whose average gift size has also decreased. It provides insights into those who may be struggling to maintain their support, allowing you to strategize on how to re-engage them effectively [QX156].
+3. **Retention by Donor Segment**: This metric examines retention rates across different gift sizes and can help you understand how various segments are performing over time. It can provide context on whether the decline in giving is a broader trend or specific to certain donor segments [CI Hub Modified FINAL LARGE DOC (1), Page 25].
+4. **Lapse Intelligence Metrics**: This includes analyzing donors who have lapsed, defined as those who have not contributed within the current analysis timeframe. By looking at pre-lapse behavioral indicators, you can identify patterns that may signal a decline in giving before it happens, allowing for proactive engagement [CI Hub Modified FINAL LARGE DOC (1), Page 25].
+5. **Bottom Segment Gift Amount Trends**: This analysis can provide insights into the trends of gift amounts among the bottom segment, helping you understand if there are consistent patterns of decline that need addressing [QX91].
+By utilizing these analytics, you can gain a comprehensive view of your donors' giving behaviors and identify those who are giving less than they used to. Blend these RFM-based analytics with engagement analytics for a better picture.</t>
+  </si>
+  <si>
+    <t>[QX137] | [QX9] | [QX136] | CI Hub Modified FINAL LARGE DOC (1) (Page 13)</t>
+  </si>
+  <si>
+    <t>To assess whether your bottom donors are at risk, you should focus on specific RFM (Recency, Frequency, Monetary Value) analytics that can provide insights into their giving behavior. Here are the key analytics to consider:
+1. **Recency Analysis**: This metric will help you understand how recently your bottom donors have made a contribution. A longer gap since their last donation may indicate a risk of disengagement. Look for trends in recency among your bottom donor segment to identify those who have not given recently [QX137].
+2. **Frequency Analysis**: Evaluate how often your bottom donors have contributed over a specific period. If their frequency of giving has decreased, it could signal that they are at risk of dropping off. This analysis can help you pinpoint which donors may need re-engagement efforts [QX136].
+3. **Monetary Value Analysis**: Assess the total amount contributed by your bottom donors. If their monetary contributions are declining, it may indicate a risk of losing these donors altogether. Understanding their giving patterns can help you strategize on how to retain them [QX9].
+4. **Annual Segment Transition Stats**: Review the transition of donors between segments over time. This can provide insights into whether your bottom donors are moving towards lower engagement or if they are at risk of becoming lapsed donors [QX136].
+5. **Concentration Ratios**: Analyze the concentration of revenue from your bottom donors. If a significant portion of your revenue is coming from a small number of bottom donors, they may be at higher risk. Understanding these ratios can help you prioritize retention strategies for this group [CI Hub Modified FINAL LARGE DOC (1), Page 13].
+By focusing on these RFM-based analytics, you can gain a clearer picture of the risk status of your bottom donors. However, to enhance your understanding, consider blending these RFM-based analytics with engagement analytics for a better picture. This will allow you to see not just the giving patterns but also how engaged these donors are with your organization.</t>
+  </si>
+  <si>
+    <t>[QX13] | [QX10] | [QX11] | CI Hub Modified FINAL LARGE DOC (1) (Page 37) | seasonal giving patterns (Page 2) | Reiley 2015 Broadcasting Suggested Donations Field Experiment (Page 19)</t>
+  </si>
+  <si>
+    <t>To assess how gift counts are trending and whether donors are giving less frequently, you should focus on the following analytics:
+1. **Gift Count Trends Among All Current Donors Analysis**: This report provides a comprehensive view of gift frequency trends for every donor who gave last year. It allows you to analyze how the number of gifts made each year has evolved over the past four fiscal years. By examining this data, you can identify which donors are increasing, maintaining, or decreasing their engagement levels [QX13].
+2. **Middle Donor Gift Count Trends Analysis**: This analysis specifically targets middle-tier individual donors whose giving frequency has declined compared to their own historical averages. It helps you track year-over-year changes in donor activity, which can be an early indicator of waning engagement among this important segment [QX11].
+3. **Gift Size Distribution + Donor Retention Cohort Analysis**: Understanding how giving patterns correlate with retention behavior across different donor segments can provide insights into whether donors are giving less frequently. This analysis helps you balance upgrade pressure with donor satisfaction, which is crucial for maintaining donor relationships [CI Hub Modified FINAL LARGE DOC (1) (Page 37)].
+4. **Seasonal Giving Patterns**: This report emphasizes the importance of tracking individual donor seasonal behavior. If a donor who typically gives during a specific time frame skips their usual gift window, it may indicate a relationship at risk. Monitoring these patterns can help you identify potential declines in engagement early on [seasonal giving patterns (Page 2)].
+5. **Constituent Intelligence Insights**: By reviewing metrics such as "Gifts (Last Full FY)", "Avg Gifts (Prior 3 FYs)", and "Last FY Count Below 3 yr Avg", you can gain a nuanced understanding of donor behavior. This analysis allows you to proactively address potential disengagement by tailoring communications to acknowledge past generosity and inquire about changes in their engagement [QX10].
+By utilizing these analytics, you can effectively determine whether donors are giving less frequently and take appropriate actions to re-engage them. Blend these RFM-based analytics with engagement analytics for a better picture.</t>
+  </si>
+  <si>
+    <t>[QX174] | [QX76] | [QX57] | CI Hub Modified FINAL LARGE DOC (1) (Page 40) | Shaker Nelson 2021 Grounded Theory Major Gift Relationships (Page 16) | Stanford PACS 2020 Community Based Orgs High Capacity Donors (Page 4)</t>
+  </si>
+  <si>
+    <t>To determine how many new donors your organization acquired last year, you should focus on the following analytics:
+1. **New Donors Last Fiscal Year**: This analytic specifically examines all new donors who made their first contribution in the last complete fiscal year. It provides insights into their giving patterns, including the number and amount of gifts they contributed, which is crucial for assessing donor retention and growth [QX174].
+2. **First-Time All Donors (10 Year) Annual Analysis**: This report tracks the long-term retention and value of new donors acquired over the last ten fiscal years. It includes annual counts of new donors, total and average first gift amounts, and retention rates, which will help you understand the scale of your new donor acquisition efforts [QX57].
+3. **Cumulative Giving Analysis**: While not directly focused on new donors, analyzing cumulative giving across the last two fiscal years can provide context on how new donors are contributing over time and their potential for future support [QX76].
+4. **Retention Hub**: This analysis can help you evaluate how well you are retaining new donors acquired in the last fiscal year, which is essential for understanding the effectiveness of your acquisition strategies [QX76].
+By reviewing these analytics, you will gain a comprehensive understanding of your new donor acquisition for the last year. Remember, blending these RFM-based analytics with engagement analytics will provide a better picture of donor behavior and retention strategies.</t>
+  </si>
+  <si>
+    <t>[QX14] | [QX52] | [QX58] | CI Hub Modified FINAL LARGE DOC (1) (Page 41) | PreventDonorAttrition (1) (Page 2)</t>
+  </si>
+  <si>
+    <t>To determine whether new donors are making a second gift, you should focus on several key RFM-based analytics that can provide insights into donor behavior and retention. Here are the specific analytics you should review:
+1. **First and Second Gift Analysis**: This analysis will help you understand the average time between a donor's first and second gifts, as well as the percentage of new donors who make a second gift. This data can indicate how quickly new donors are engaging with your organization and whether your stewardship efforts are effective in encouraging repeat donations [QX14].
+2. **Retention Rates by Acquisition Year**: Examine the retention rates of new donors segmented by their acquisition year. This will allow you to see how many of these donors are returning for a second gift and whether there are trends over time that indicate improvements or declines in retention [QX52].
+3. **Cohort Analysis of First-Time Donors**: Conduct a cohort analysis focusing on first-time donors to track their giving behavior over time. This will help you identify patterns in their likelihood to make a second gift and can inform your cultivation strategies [QX58].
+4. **Donor Lifecycle Trends**: Analyze the overall donor lifecycle, paying special attention to the share of new donors who are retained or renewed each year. This will give you a broader view of how new donors are performing in terms of making subsequent gifts [PreventDonorAttrition (1)].
+5. **Upgrade Rates**: Look at the upgrade rates of new donors who have made a second gift. This can provide insights into whether your messaging and stewardship efforts are effectively encouraging larger subsequent gifts [QX14].
+By focusing on these analytics, you can gain a clearer picture of how new donors are engaging with your organization and whether they are making a second gift. Remember to blend these RFM-based analytics with engagement analytics for a better picture, as engagement data can provide additional context to donor behavior.</t>
+  </si>
+  <si>
+    <t>[QX26] | [QX15] | [QX14] | CI Hub Modified FINAL LARGE DOC (1) (Page 45)</t>
+  </si>
+  <si>
+    <t>To assess whether your second-time donors are making a third gift, you should focus on the **Second to Third Gift Retention Analysis**. This analysis is specifically designed to track the transition of donors from their second to their third gift, which is a critical stage in fostering long-term donor relationships. 
+Hereâ€™s how you can utilize this analysis effectively:
+1. **Retention Metrics**: The analysis will provide you with the percentage of donors who make a third gift after their second. This is crucial for understanding how well you are retaining your donors at this pivotal point in their giving journey [QX15].
+2. **Segmentation by Value Tiers**: By segmenting your donors into value tiers (Top, Middle, Bottom) based on the combined amount of their first two gifts, you can gain insights into which segments are more likely to convert to a third gift. This can help tailor your follow-up strategies [QX15].
+3. **Timing Insights**: The analysis also examines how quickly donors move from their second to third gift. Understanding the timing can help you identify patterns and optimize your engagement strategies to encourage quicker conversions [QX15].
+4. **Behavioral Patterns**: Look for behaviors such as whether donors upgrade their giving on the third donation. This can provide insights into donor satisfaction and the effectiveness of your stewardship efforts [QX15].
+5. **Long-Term Trends**: Tracking these metrics over time will allow you to measure improvements in conversion rates and identify successful strategies that strengthen donor retention [QX14].
+By focusing on the **Second to Third Gift Retention Analysis**, you can gain a comprehensive view of your second-time donors' behavior and make informed decisions to enhance your donor retention strategies. 
+Blend these RFM-based analytics with engagement analytics for a better picture. This will provide a more holistic view of your donor relationships and help you identify additional opportunities for engagement and retention.</t>
+  </si>
+  <si>
+    <t>[QX74] | [QX51] | [QX57] | CI Hub Modified FINAL LARGE DOC (1) (Page 19)</t>
+  </si>
+  <si>
+    <t>To assess your first-year donor retention rate, you should focus on the following analytics available in your Constituent Intelligence Hub:
+1. **First Time Donors by Month and Retention**: This analysis will provide you with insights into how many first-time donors are retained after their initial contribution. It tracks retention rates over the first year and can help you identify trends in donor loyalty [QX74].
+2. **Retention Rates by Acquisition Year**: This metric highlights how many first-time donors are retained in the first fiscal year and beyond. It also provides raw counts and retention rates, allowing you to evaluate the effectiveness of your onboarding strategies and identify any areas needing improvement [QX51].
+3. **Cumulative Value of Gifts from First-Time Donors**: This analysis measures the total contributions made by first-time donors over their first three years, segmented by retained donors. It helps quantify the lifetime value of new donor acquisition, which is crucial for understanding the impact of your retention efforts [QX57].
+4. **Donor Retention by Acquisition Season**: This analytic can reveal how retention rates vary by the season in which donors were acquired. For instance, you might find that donors acquired during specific campaigns retain at higher rates than those acquired during others, which can inform your future acquisition strategies [CI Hub Modified FINAL LARGE DOC (1), Page 19].
+By reviewing these analytics, you can gain a comprehensive understanding of your first-year donor retention rate and identify strategies to enhance donor loyalty. Remember, blending these RFM-based analytics with engagement analytics will provide a better picture of your donor retention efforts.</t>
+  </si>
+  <si>
+    <t>[QX10] | [QX76] | [QX27] | seasonal giving patterns (Page 3) | CI Hub Modified FINAL LARGE DOC (1) (Page 17)</t>
+  </si>
+  <si>
+    <t>To determine when your organization acquires the most new donors throughout the year, you should focus on analyzing **Seasonal Giving Patterns**. This analysis will help you understand the timing of donor acquisition and the factors influencing these trends.
+1. **Seasonal Giving Patterns**: Review the monthly and quarterly patterns of donor acquisition. Different nonprofit sectors experience distinct seasonal peaks, such as higher education benefiting from reunion weekends in spring and fall, or healthcare organizations seeing increased giving during gala seasons. By aligning your major campaigns with these institutional cycles, you can identify optimal times for donor acquisition [Seasonal Giving Patterns (Page 3)].
+2. **Acquisition Year and Growth Ranking**: Utilize the data that includes donors who have made a gift within the last two fiscal years. This analysis will provide insights into the acquisition year, total giving in their first year, and last gift date. Understanding these metrics will help you pinpoint when new donors are most likely to engage with your organization [QX76].
+3. **Donor Cohort Analysis**: Examine how many new donors convert to sustained multi-year giving and the rates for each cohort over time. This will help you identify which acquisition years have yielded the best long-term results and when your outreach efforts are most effective [QX27].
+4. **Retention Campaign Timing**: Consider the timing of your retention campaigns, as effective outreach can significantly impact donor acquisition. Understanding when donors are most receptive can help you refine your strategies and improve acquisition rates [CI Hub Modified FINAL LARGE DOC (1) (Page 17)].
+By focusing on these RFM-based analytics, you can gain valuable insights into your donor acquisition patterns. However, to get a more comprehensive view, **blend these RFM-based analytics with engagement analytics for a better picture**. This will allow you to understand not just when donors are acquired, but also how to effectively engage them moving forward.</t>
+  </si>
+  <si>
+    <t>[QX74] | [QX26] | [QX46] | CI Hub Modified FINAL LARGE DOC (1) (Page 26)</t>
+  </si>
+  <si>
+    <t>To analyze how your new donor acquisition trends have changed over the past 10 years, you should focus on several key RFM-based analytics that can provide insights into donor behavior and retention patterns. Here are the specific analytics you should consider:
+1. **First Time Donors by Month and Retention**: This analytic will help you track the number of new donors acquired each month over the past decade and their subsequent retention rates. By examining this data, you can identify trends in acquisition and how effectively you are retaining these new donors over time [QX74].
+2. **13-Month Retention Rates**: Evaluating your 13-month retention rates year over year will provide insights into how well you are maintaining relationships with new donors. This metric is crucial for understanding the effectiveness of your onboarding and engagement strategies for new donors [QX26].
+3. **Average Second Gift Amounts**: Analyzing the average amounts of second gifts from new donors can indicate the level of commitment and satisfaction among your new donor base. If this amount is increasing, it may suggest that your acquisition strategies are successfully converting new donors into more engaged supporters [QX26].
+4. **New Donor Onboarding Monitor**: This analytic can help you assess the effectiveness of your onboarding processes for new donors. By reviewing the data, you can identify any gaps or areas for improvement in how you engage new donors right after acquisition [QX26].
+5. **Donor Lifecycle Data**: Utilize the donor lifecycle analytics to interpret patterns in your new donor acquisition and retention. This data will provide a comprehensive view of how your new donor base has evolved over the years, including retention rates and acquisition flows [CI Hub Modified FINAL LARGE DOC (1), Page 26].
+By focusing on these RFM-based analytics, you can gain a clearer understanding of your new donor acquisition trends over the past decade. Remember, blending these RFM-based analytics with engagement analytics will provide a better picture of your overall donor engagement and retention strategies.</t>
+  </si>
+  <si>
+    <t>[QX91] | [QX15] | [QX170] | CI Hub Modified FINAL LARGE DOC (1) (Page 5)</t>
+  </si>
+  <si>
+    <t>To identify which donors are ready for a higher ask, you should focus on several key RFM (Recency, Frequency, Monetary Value) analytics that can provide insights into donor behavior and potential for increased giving. Here are the specific analytics you should consider:
+1. **3rd Gift Conversion Rate**: This metric tracks the movement of donors from their first to second and then to their third gift. By analyzing this rate, you can identify which segments are most likely to upgrade their giving. A higher conversion rate indicates that donors are engaged and may be ready for a higher ask [QX15].
+2. **Upgrade Rate**: This metric helps you understand how many donors are moving to higher giving tiers. By monitoring the upgrade rate, you can pinpoint donors whose giving potential is growing and who may be receptive to a higher ask [QX15].
+3. **Average and Median Gift Amounts**: Reviewing the average and median amounts given at each stage of the donor journey can help you identify which donors are contributing at levels that suggest they might be ready to increase their support. If you see a trend of increasing gift amounts, it may indicate readiness for a higher ask [QX15].
+4. **Retention Rates**: Focus on the retention rates of your most engaged segments. If certain donor cohorts are showing improved retention, they are likely more committed and may be more open to increasing their contributions [QX170].
+5. **Donor Tenure and Channel Segmentation**: Segmenting your donors by tenure and the channels through which they give can provide insights into their loyalty and engagement levels. Longer-tenured donors or those who give through multiple channels may be more likely to respond positively to a higher ask [QX91].
+By analyzing these RFM-based metrics, you can better understand which donors are primed for a higher ask. Remember to blend these RFM-based analytics with engagement analytics for a better picture of donor readiness. This comprehensive approach will allow you to tailor your outreach and maximize the potential for increased giving.</t>
+  </si>
+  <si>
+    <t>[QX159] | [QX97] | [QX158] | upgrade potential analysis (Page 2) | CI Hub Modified FINAL LARGE DOC (1) (Page 59)</t>
+  </si>
+  <si>
+    <t>To identify your best upgrade prospects for major gifts, you should focus on the following RFM-based analytics:
+1. **Top Segment Stable-Target Increase**: This analytic identifies upgrade candidates from your top-segment donor pool who have consistently given at a stable level over the past two years. It assesses historical giving data to highlight donors who have maintained or increased their contributions, making them prime candidates for major gift solicitations [QX159].
+2. **Bottom Segment Stable-Target Increase**: While this analysis focuses on the bottom-segment donor pool, it can still provide valuable insights. It identifies donors who have shown stable giving patterns and may be on the verge of upgrading. Understanding these donors can help you cultivate relationships that could lead to major gifts in the future [QX158].
+3. **Upgrade Potential Analysis**: This analysis helps you pinpoint the most promising donor advancement opportunities by evaluating current giving levels against tier benchmarks. It categorizes donors based on their performance and identifies those who are close to moving up a tier, which can be crucial for targeting major gift asks [Upgrade Potential Analysis (Page 2)].
+4. **Donor Upgrade Pipeline**: This analytic tracks the movement of donors through different giving tiers, allowing you to see who is progressing towards major gifts. By regularly reviewing this pipeline, you can focus your efforts on those who are most likely to upgrade their support [QX97].
+5. **Retention Hub**: While primarily focused on retention, this analytic can provide insights into donor satisfaction and engagement levels, which are critical when considering major gift prospects. Understanding which donors are likely to remain engaged can help you tailor your approach for major gift solicitations [CI Hub Modified FINAL LARGE DOC (1) (Page 59)].
+By leveraging these RFM-based analytics, you can effectively identify and prioritize your best upgrade prospects for major gifts. Remember to blend these RFM-based analytics with engagement analytics for a better picture of your donor relationships and potential.</t>
+  </si>
+  <si>
+    <t>[QX164] | [QX16] | [QX161] | CI Hub Modified FINAL LARGE DOC (1) (Page 41) | Shaker Nelson 2021 Grounded Theory Major Gift Relationships (Page 32) | Nyman Pilbeam Baines Maklan 2016 Transformational Gifts Roles Accepted Manuscript (Page 3)</t>
+  </si>
+  <si>
+    <t>To understand how long it takes for a donor to reach the major gift level, you should focus on the following analytics:
+1. **Average Tenure to Major Gift Detail**: This analysis provides a detailed breakdown of the donor journey from their first gift to their first major gift, specifically focusing on gifts that meet or exceed a predefined threshold for major giving. It constructs a chronological timeline of gifts for each donor, allowing you to identify key milestones in their giving history, including the time it takes for donors to reach major gift status [QX164].
+2. **Average Tenure to Top Level Donor Analysis**: This analysis tracks the progression of donors from their initial contribution to the moment they make a top-level or major gift. It captures the number of gifts it took before they became a major donor and the total amount contributed up to that point. This will help you understand the typical duration it takes for constituents to reach that key giving threshold [QX16].
+3. **Donor Tenure Distribution by Initial Segment**: This analytic examines how long donors remain active based on the segment they belonged to during their first year of giving. It provides insights into the average tenure of donors in different segments, which can help you understand the retention patterns and how they relate to the time taken to reach major gift status [QX161].
+4. **Tenure-Based Stewardship Tracks**: By analyzing tenure patterns, you can redesign your onboarding and stewardship strategies. Understanding the typical time it takes for donors to reach major gift levels can inform how you cultivate relationships with donors at different stages of their giving journey [CI Hub Modified FINAL LARGE DOC (1), Page 41].
+By leveraging these RFM-based analytics, you can gain insights into the donor journey and the time it typically takes for donors to reach major gift levels. Blend these RFM-based analytics with engagement analytics for a better picture.</t>
+  </si>
+  <si>
+    <t>[QX153] | [QX99] | [QX155] | CI Hub Modified FINAL LARGE DOC (1) (Page 18) | Stanford PACS 2020 Community Based Orgs High Capacity Donors (Page 21)</t>
+  </si>
+  <si>
+    <t>To identify donors who started small and have transitioned into major donors, you should focus on several key RFM-based analytics that can provide insights into their giving patterns and potential for upgrades. Here are the specific analytics and metrics you should consider:
+1. **Growth &amp; Upgrade Pipeline**: This analysis will help you identify donors whose gift sizes are increasing over time. By examining the trends in their giving, you can pinpoint those who have moved from smaller contributions to larger ones, indicating a readiness for major donor conversations [QX153].
+2. **Donor Upgrade Pipeline**: This report focuses on identifying donors whose largest gifts are at or above certain percentiles compared to middle-segment donors. By reviewing this data, you can find individuals who may be ready for an upgrade conversation based on their giving history and current engagement levels [QX99].
+3. **Recency Analysis**: Look at the recency of donations from these donors. A donor who has recently made a gift, especially after a period of smaller contributions, may be signaling increased engagement and interest in your organization. This is crucial for understanding their current relationship status [CI Hub Modified FINAL LARGE DOC (1), Page 18].
+4. **Frequency Metrics**: Analyze how often these donors have contributed over the past year. A shift from infrequent to more regular giving can indicate a growing commitment to your organization, making them prime candidates for major donor cultivation [QX155].
+5. **Monetary Value Trends**: Review the total monetary contributions from these donors over time. Tracking the increase in their total giving can help you identify those who have the potential to become major donors, especially if their contributions have significantly increased in recent years [Stanford PACS 2020 Community Based Orgs High Capacity Donors, Page 21].
+By focusing on these RFM-based analytics, you can effectively identify and engage with donors who have shown a trajectory from small to major gifts. Remember to blend these RFM-based analytics with engagement analytics for a better picture of their readiness and potential for further contributions.</t>
+  </si>
+  <si>
+    <t>[QX22] | [QX149] | [QX14] | seasonal giving patterns (Page 3) | CI Hub Modified FINAL LARGE DOC (1) (Page 9)</t>
+  </si>
+  <si>
+    <t>To analyze overall upgrade and downgrade patterns among your donors, you should focus on several key RFM-based analytics that will provide insights into donor behavior and transitions. Here are the specific analytics you should consider:
+1. **Donor Upgrade Analysis**: This analytic examines how many donors have historically upgraded their annual giving by 25% or more compared to their initial year. It tracks the timeframes before these upgrades occurred and segments donors into categories such as "Top," "Middle," and "Bottom" based on their first-year contributions. Key metrics include the percentage of donors who upgrade and the average time to upgrade, which can help you identify trends in donor mobility and the effectiveness of your stewardship strategies [QX149].
+2. **Multi-Year Donor Upgrade Analysis**: This analysis focuses on multi-year donors who have increased their giving by at least 20%. It provides insights into how these groups evolve over time and the characteristics of donors who upgrade. Understanding the average upgrade percentage and the time it takes for upgrades can inform your engagement strategies and highlight potential areas for improvement [QX149].
+3. **Retention Hub**: This analytic allows you to assess the proportion of donors who upgraded, downgraded, or maintained their tier. By examining the average and median gift totals for each group, you can spot trends in retention among top donors and identify opportunities for middle-tier donors to move up. This analysis is crucial for understanding the effectiveness of your stewardship and upgrade strategies over time [QX22].
+4. **Gift Frequency and Timing Analysis**: This analysis looks at the frequency of gifts and the timing of second gifts, including the percentage of donors who increased their gift on their second donation. It can help you identify which segments are most likely to return and how quickly they do so, providing insights into the effectiveness of your follow-up and engagement efforts [QX14].
+5. **Seasonal Giving Patterns**: Understanding seasonal trends can also inform your analysis of upgrades and downgrades. By examining whether seasonal peaks are driven by many small contributions or fewer large gifts, you can identify upgrade opportunities and monitor potential concentration risks among your donor base [Seasonal Giving Patterns, Page 3].
+By reviewing these analytics, you can gain a comprehensive understanding of your donors' upgrade and downgrade patterns. Remember to blend these RFM-based analytics with engagement analytics for a better picture of donor behavior and to refine your outreach strategies effectively.</t>
+  </si>
+  <si>
+    <t>[QX97] | [QX96] | [QX99] | upgrade potential analysis (Page 2) | CI Hub Modified FINAL LARGE DOC (1) (Page 60)</t>
+  </si>
+  <si>
+    <t>To determine if your middle donors are receiving upgrade prospect lists, you should focus on the **Middle Segment Donor Upgrade Prospect List Analysis**. This analysis is specifically designed to identify promising upgrade candidates from your mid-level donor pool by examining their recent giving behavior and contributions over the past two fiscal years.
+Here are the key analytics you should review:
+1. **Middle Segment Donor Upgrade Prospect List**: This report highlights donors who are at the top end of the middle donor range and are approaching the minimum threshold for your top donor segment. It identifies those who have made significant gifts recently, which indicates high upgrade potential [QX97].
+2. **Review Frequency**: Ensure that this analysis is reviewed regularlyâ€”ideally quarterly. This will help you capture new prospects as giving patterns emerge and ensure that your middle donors are being actively considered for upgrades [QX96].
+3. **Follow-Up Actions**: Check if specific follow-up actions are being assigned to the highlighted donors, such as personalized thank-you calls or tailored upgrade solicitations. This is crucial for nurturing relationships and encouraging upgrades [QX96].
+4. **Metrics Tracking**: Monitor the success of the upgrade efforts by tracking metrics such as the percentage of identified prospects who increase their giving and the overall revenue lift from this cohort. This will provide insights into the effectiveness of your upgrade strategies [QX99].
+5. **Upgrade Potential Analysis**: Utilize the Upgrade Potential Analysis to identify which middle donors show genuine upgrade potential. This analysis helps in focusing your cultivation efforts on the most promising candidates, thereby enhancing your overall donor advancement strategy [QX99].
+By focusing on these analytics, you can ensure that your middle donors are being effectively targeted for upgrades. Remember to blend these RFM-based analytics with engagement analytics for a better picture of your donor relationships.</t>
+  </si>
+  <si>
+    <t>[QX69] | [QX68] | [QX66] | CI Hub Modified FINAL LARGE DOC (1) (Page 25)</t>
+  </si>
+  <si>
+    <t>To identify which lapsed donors returned this year, you should focus on the following RFM-based analytics:
+1. **Recapture History Analysis**: This analysis will provide insights into the number of lapsed donors who have returned, including the fiscal years of their pre-lapse and recapture gifts. It will also detail the months lapsed and the giving amounts before and after recapture. This data is crucial for assessing whether their re-engagement is sustained or at risk [QX66].
+2. **Reactivation Rate**: This metric measures the percentage of lapsed donors who have returned to giving. It will help you quantify the success of your reactivation efforts and understand the overall effectiveness of your strategies in bringing back lapsed donors [CI Hub Modified FINAL LARGE DOC (1), Page 25].
+3. **Time from Lapse to Reactivation**: Understanding how long donors typically remain lapsed before returning can provide insights into the effectiveness of your outreach strategies. This metric can help you refine your timing for future re-engagement efforts [CI Hub Modified FINAL LARGE DOC (1), Page 25].
+4. **Post-Reactivation Retention**: This metric compares the performance of reactivated donors to newly acquired donors. It can help you assess the long-term value of reactivated donors and inform your stewardship strategies moving forward [CI Hub Modified FINAL LARGE DOC (1), Page 25].
+5. **Donor Upgrade Pipeline**: By analyzing the giving levels of recently recaptured donors, you can identify those who may be at risk of lapsing again or those who have the potential to upgrade their giving. This will allow you to prioritize outreach and tailor stewardship efforts accordingly [QX68].
+By focusing on these analytics, you can gain a comprehensive understanding of your lapsed donors who returned this year and develop strategies to enhance their engagement and giving levels. Remember to blend these RFM-based analytics with engagement analytics for a better picture.</t>
+  </si>
+  <si>
+    <t>[QX66] | [QX65] | [QX67] | CI Hub Modified FINAL LARGE DOC (1) (Page 39)</t>
+  </si>
+  <si>
+    <t>To identify which segment your recaptured donors are coming from, you should focus on the **Recent Middle Donor Recaptures Analysis**. This analysis provides a comprehensive view of donors who were previously classified as middle-level based on your organization's giving thresholds, lapsed for at least a year, and then returned with a new gift in a recent fiscal year. It includes detailed information such as the number of recapture events, the fiscal years of pre-lapse and recapture gifts, and the months lapsed, which will help you pinpoint the specific segments of donors that are re-engaging with your organization [QX66].
+Additionally, you can utilize the insights from the **Recent Donor Recaptures** analysis to assess the behavior of donors who were previously at the bottom tier. This will allow you to see which strategies have been effective in re-engaging these at-risk donors and whether their giving levels have increased or been maintained upon their return [QX67].
+By analyzing these segments, you can tailor your outreach and stewardship strategies accordingly, ensuring that you are effectively engaging with the right donor segments to enhance retention and increase giving levels [QX65].
+In summary, focus on the following analytics:
+1. **Recent Middle Donor Recaptures Analysis** - to identify middle-level donor recaptures.
+2. **Recent Donor Recaptures Analysis** - to understand the behavior of bottom-segment donors who have been recaptured.
+These insights will provide a clearer picture of your recaptured donor segments and inform your retention strategies.</t>
+  </si>
+  <si>
+    <t>[QX162] | [QX47] | [QX69] | CI Hub Modified FINAL LARGE DOC (1) (Page 25)</t>
+  </si>
+  <si>
+    <t>To analyze your 10-year recapture history effectively, you should focus on several key RFM-based analytics that will provide insights into donor behavior over time. Here are the specific analytics you should consider:
+1. **All Donor Recaptures (10yr)**: This analytic will give you a comprehensive view of how many lapsed donors have returned to giving over the past decade. It will help you understand the overall effectiveness of your reactivation strategies and the trends in donor recapture [QX69].
+2. **Reactivation Rate**: This metric measures the percentage of lapsed donors who have returned to active giving. Itâ€™s crucial for assessing the success of your reactivation efforts and understanding how well you are engaging lapsed donors [CI Hub Modified FINAL LARGE DOC (1), Page 25].
+3. **Time from Lapse to Reactivation**: This analytic will provide insights into how long donors typically remain lapsed before returning. Understanding this timeline can help you refine your outreach strategies and timing for re-engagement efforts [CI Hub Modified FINAL LARGE DOC (1), Page 25].
+4. **Reactivation Success by Lapse Duration**: This metric allows you to analyze whether donors who lapsed for shorter periods respond differently than those who have been lapsed for longer durations. This can inform targeted strategies for different segments of lapsed donors [CI Hub Modified FINAL LARGE DOC (1), Page 25].
+5. **Post-Reactivation Retention**: This analytic compares the retention rates of reactivated donors to those of newly acquired donors. It can provide valuable insights into the long-term value of reactivated donors and help you assess the effectiveness of your reactivation strategies [CI Hub Modified FINAL LARGE DOC (1), Page 25].
+By examining these analytics, you will gain a clearer picture of your 10-year recapture history and the effectiveness of your donor reactivation strategies. Remember, blending these RFM-based analytics with engagement analytics will provide a better picture of your overall donor engagement and retention efforts.</t>
+  </si>
+  <si>
+    <t>[QX158] | [QX31] | [QX159] | CI Hub Modified FINAL LARGE DOC (1) (Page 5) | upgrade potential analysis (Page 2)</t>
+  </si>
+  <si>
+    <t>To effectively score your top donors for risk and opportunity, you should focus on several key RFM-based analytics that will provide insights into their giving behavior and potential for future contributions. Here are the recommended analytics to consider:
+1. **Active Top Donor 2-Year Frequency Trend Score**: This metric will help you understand the frequency of donations from your top donors over the past two years. A declining frequency could indicate a risk of disengagement, while stable or increasing frequency suggests a strong relationship that can be further cultivated [QX31].
+2. **Upgrade Potential Analysis**: This analysis identifies donors who are on the cusp of moving to a higher giving tier. By evaluating their current giving levels, average gift size, and the amount needed to reach the next tier, you can pinpoint those who have the potential for increased contributions. This is crucial for focusing your efforts on donors who are likely to respond positively to targeted engagement strategies [upgrade potential analysis (Page 2)].
+3. **Donor Segmentation**: Utilize the segmentation of your donor base into categories such as 'Stable Donors' who are eligible for increases. This segmentation allows you to tailor your outreach and engagement strategies based on the specific characteristics and giving patterns of each group [QX159].
+4. **Scoring System for Donor Performance**: Implement a scoring system that categorizes donors based on their giving history, such as those who have maintained or increased their giving. This will help you identify which donors are already inclined to give more and can be targeted for further engagement [QX158].
+5. **Strategic Risk Assessment**: Regularly assess your donor portfolio for red flags, such as declining gift frequency or a growing dependency on a small percentage of donors for revenue. This will help you identify potential risks in your donor base and take proactive measures to mitigate them [CI Hub Modified FINAL LARGE DOC (1) (Page 5)].
+By blending these RFM-based analytics with engagement analytics, you can gain a more comprehensive understanding of your top donors' behaviors and motivations, allowing you to craft more effective fundraising strategies.</t>
+  </si>
+  <si>
+    <t>[QX172] | [QX33] | [QX166] | CI Hub Modified FINAL LARGE DOC (1) (Page 6)</t>
+  </si>
+  <si>
+    <t>To effectively score middle donors, you should focus on several key analytics that will provide insights into their giving patterns and engagement levels. Here are the specific analytics you should consider:
+1. **Active Middle Donor 5-Year Amount Score Summary**: This analysis evaluates your middle-tier donors based on their giving patterns over the last five fiscal years. It categorizes donors by coded scores that reflect their annual giving amounts, identifying trends such as increases, decreases, lapses, or new engagement. This summary will help you understand the overall health of your middle donor segment and identify those who may need targeted engagement strategies [QX33].
+2. **Middle Segment Donor Loyalty Analysis**: This analytic focuses on the long-term loyalty of donors within the Middle Segment. It examines their consistency in giving over multiple years and identifies how many years they have contributed at a higher, Top Segment level. Key metrics include the total number of years of contribution and the current streak of consecutive contributions, which can help you identify loyal donors who may be ripe for upgrades [QX166].
+3. **Segment-Specific Year-Over-Year Metrics**: For middle donors, you should monitor upgrade patterns, retention rates, and acquisition into this segment. This analysis is crucial as the middle level often represents your best upgrade pipeline and provides stability between major gifts. Understanding these metrics will allow you to tailor your engagement strategies effectively [CI Hub Modified FINAL LARGE DOC (1), Page 6].
+4. **Donor Segmentation Analysis**: By segmenting your donors based on their giving levels, you can better understand where they fall within your organization's hierarchy of donor engagement. This will help you design targeted communication strategies and set appropriate fundraising goals for each segment, particularly focusing on converting Middle Max donors into Top Min donors [QX172].
+5. **Retention Hub**: While not explicitly mentioned in the provided sources, tracking retention rates for your middle donors is essential. A decline in retention can significantly impact your revenue, so understanding the retention trends within this segment will help you identify areas for improvement and engagement [CI Hub Modified FINAL LARGE DOC (1), Page 6].
+By utilizing these analytics, you can develop a comprehensive scoring system for your middle donors that not only reflects their past giving behavior but also informs your future engagement strategies. Remember to blend these RFM-based analytics with engagement analytics for a better picture.</t>
+  </si>
+  <si>
+    <t>[QX167] | [QX172] | [QX91] | CI Hub Modified FINAL LARGE DOC (1) (Page 35)</t>
+  </si>
+  <si>
+    <t>To effectively analyze donor scores across your entire donor base, you should focus on the following RFM-based analytics:
+1. **Bottom Segment Donor Loyalty Analysis**: This analytic provides insights specifically into the loyalty of donors categorized in the Bottom Segment. It tracks giving patterns, including the total annual giving and the streak of consecutive years a donor has contributed. This can help you identify trends and potential upgrade opportunities within this segment [QX167].
+2. **Donor Segmentation Analysis**: Understanding the hierarchy of donor engagement levels is crucial. This analysis allows you to see where donors fall within your organization's giving levels, from the Bottom Segment to the Top Segment. By reviewing these segments, you can tailor your engagement strategies and identify potential pathways for upgrading donors [QX172].
+3. **Gift Size Distribution Analytics**: This analytic will show you the distribution of gift sizes across your donor base. By examining percentile values, you can identify clear upgrade pathways and understand how your bottom-tier donors compare to mid-tier donors. This can reveal significant overlap that may indicate opportunities for upgrading donors [CI Hub Modified FINAL LARGE DOC (1) (Page 35)].
+4. **Annual Review of Bottom Donor Metrics**: Regularly reviewing metrics such as the number of bottom donors, total giving from this group, and average and median gift amounts will help you monitor the health of your entry-level donor pipeline. This analysis can inform your acquisition and retention strategies, ensuring you are aware of any trends that may require action [QX91].
+5. **Retention Hub**: While not explicitly mentioned in the provided sources, focusing on donor retention metrics is essential, especially given the declining overall donor retention rates. Understanding how different segments are performing can help you strategize effectively to maintain and grow your donor base [CI Hub Modified FINAL LARGE DOC (1) (Page 35)].
+By utilizing these RFM-based analytics, you can gain a comprehensive view of your donor scores. However, to enhance your understanding, consider blending these RFM-based analytics with engagement analytics for a better picture. This will provide a more holistic view of donor behavior and engagement levels.</t>
+  </si>
+  <si>
+    <t>[QX172] | [QX92] | [QX49] | CI Hub Modified FINAL LARGE DOC (1) (Page 6)</t>
+  </si>
+  <si>
+    <t>To define your segments and thresholds effectively, you should focus on analyzing your donor data through the lens of RFM metrics (Recency, Frequency, Monetary Value). Here are the key analytics you should consider:
+1. **Active Top Segment Analysis**: This involves tracking retention rates, average gift trends, and gift frequency for your highest-capacity donors. Understanding these metrics will help you identify the thresholds that define your top segment, as a decline in retention among these donors can significantly impact your revenue [CI Hub Modified FINAL LARGE DOC (1) (Page 6)].
+2. **Active Middle Segment Analysis**: Monitor upgrade patterns, retention rates, and acquisition into this segment. The middle segment often serves as a crucial upgrade pipeline, and analyzing these metrics will help you establish clear definitions and thresholds for this group [CI Hub Modified FINAL LARGE DOC (1) (Page 6)].
+3. **Small-Dollar Segment Analysis**: Focus on participation trends, retention rates, and acquisition effectiveness within this segment. While individual gifts may be smaller, understanding their behavior can help you define thresholds for sustainability and future upgrade candidates [CI Hub Modified FINAL LARGE DOC (1) (Page 6)].
+4. **Segmentation Strategy Evaluation**: Utilize insights from your segmentation to develop targeted strategies. For example, you can create personalized moves management plans for High Prospects and tailored stewardship journeys for Emerging Prospects. This will help you refine your segment definitions based on donor behavior and engagement [QX49].
+5. **Year-Over-Year Metrics**: Track increases in top-segment retention, total dollars raised, and the movement of donors into higher giving brackets year over year. This longitudinal analysis will provide clarity on how your segments evolve and help you adjust your definitions accordingly [QX92].
+By focusing on these RFM-based analytics, you can establish clear segment definitions and thresholds that align with your fundraising goals. Remember to blend these RFM-based analytics with engagement analytics for a better picture.</t>
+  </si>
+  <si>
+    <t>[QX167] | [QX169] | [QX172] | CI Hub Modified FINAL LARGE DOC (1) (Page 26)</t>
+  </si>
+  <si>
+    <t>To understand your raw segmentation data effectively, you should focus on the following analytics and reports within your organization:
+1. **Segmentation Break Points Analysis**: This report provides a detailed view of the thresholds that categorize your donors into segments (Bottom, Middle, and Top). By examining the "Thresholds" table, you can see how donation amounts are distributed across these segments, which is crucial for understanding the financial contributions from different donor levels [QX172].
+2. **Segment Migration Detail**: This report tracks the year-over-year migration of donors across segments over the last seven fiscal years. It will help you identify patterns of retention, upgrades, and lapses among your donors. This analysis is essential for understanding how your donor segments evolve over time and can provide insights into the effectiveness of your engagement strategies [QX169].
+3. **Donor Loyalty Analysis by Segment**: This analysis focuses on the Bottom Segment donors, measuring metrics such as donor retention rates and the number of donors transitioning to higher tiers. Regularly assessing these metrics will allow you to gauge the effectiveness of your engagement strategies and adjust your approaches as needed [QX167].
+4. **Donor Lifecycle Data**: While this is more of a strategic interpretation framework, it provides general sector performance ranges that can serve as reference points for your segmentation data. Understanding these benchmarks can help you interpret your organization's actual rates by segment and identify areas for improvement [CI Hub Modified FINAL LARGE DOC (1) (Page 26)].
+By reviewing these analytics, you will gain a comprehensive understanding of your raw segmentation data, which will inform your strategies for donor engagement and retention. Remember, blending these RFM-based analytics with engagement analytics will provide a better picture of your donor landscape.</t>
+  </si>
+  <si>
+    <t>[QX167] | [QX141] | [QX137] | CI Hub Modified FINAL LARGE DOC (1) (Page 82)</t>
+  </si>
+  <si>
+    <t>To understand the probabilities of donors transitioning between segments, you should focus on specific RFM-based analytics that provide insights into donor behavior and segment dynamics. Here are the key analytics to consider:
+1. **Transition Analysis**: This analysis will help you evaluate how many donors remain in their current segment, upgrade to a higher tier, downgrade, or lapse entirely. Key metrics to track include:
+   - Maintain/Transition to Top %
+   - Transition to Middle %
+   - Transition to Bottom %
+   - Transition to Lapsed % 
+   This will allow you to pinpoint which segments require more focused stewardship and identify areas where your fundraising investments are effective or need innovation [QX137].
+2. **Donor Loyalty Analysis by Segment**: This analysis focuses on loyal Bottom Segment donors and measures the success of engagement strategies. You can establish metrics such as increased donor retention rates in the Bottom Segment and the number of donors transitioning to higher tiers. Regular assessments will help gauge the effectiveness of your strategies and adjust them as needed [QX167].
+3. **Cohort Analysis**: This approach allows you to segment your portfolios and set intervention thresholds based on donor behavior. By tracking improvements in retention rates and increases in donors upgrading segments, you can develop targeted communications and re-engagement campaigns for specific tenure bands with high lapse rates [QX141].
+4. **Retention Probability and Upgrade Probability**: These metrics are crucial for evaluating the health of your donor pipeline. Retention Probability indicates the likelihood that a donor stays in their current tier, while Upgrade Probability reflects the chance they move to a higher giving tier. Monitoring these probabilities will provide insights into donor engagement and potential risks [CI Hub Modified FINAL LARGE DOC (1) (Page 82)].
+5. **Periodic Review of Segment-Level Transitions**: Schedule regular reviews of segment-level transitions as part of your Constituent Intelligence routines. This will help you stay ahead of campaign planning and stewardship strategy sessions, ensuring that you are responsive to the dynamics within your donor segments [QX137].
+By focusing on these RFM-based analytics, you can gain a clearer picture of donor transitions between segments. Remember to blend these RFM-based analytics with engagement analytics for a better picture of donor behavior and engagement strategies.</t>
+  </si>
+  <si>
+    <t>[QX74] | [QX26] | [QX167] | CI Hub Modified FINAL LARGE DOC (1) (Page 30)</t>
+  </si>
+  <si>
+    <t>To understand the lifetime value of different donor cohorts, you should focus on several key analytics that will provide insights into donor behavior and retention over time. Here are the specific analytics you should consider:
+1. **Cohort Analysis**: This is essential for understanding how different groups of donors (cohorts) perform over time. By analyzing cohorts based on their acquisition year, quarter, or month, you can track their retention rates and revenue generation. Look specifically at the **Year 1 â†’ Year 2 Retention Rate**, which indicates how many first-year donors continue to give in their second year. This metric is crucial for assessing the quality of your acquisition strategies and understanding the potential lifetime value of these donors [CI Hub Modified FINAL LARGE DOC (1), Page 30].
+2. **First-Time Donor 13-Month Retention Analysis**: This analysis will help you evaluate how effectively you convert first-time donors into repeat donors within a critical 13-month window. By examining the percentage of new donors who make a second gift, you can gauge the initial engagement and potential lifetime value of these donors. This analysis also segments donors by gift size, allowing you to see how retention varies across different giving levels [QX26].
+3. **Bottom Segment Donor Loyalty Analysis**: Understanding the loyalty of donors in the Bottom Segment can provide insights into their giving patterns and potential for future contributions. This analysis tracks the total annual giving and consecutive years of contributions, which can help identify trends and opportunities for moving these donors into higher giving tiers. Recognizing upward movement can signal potential for increased engagement and lifetime value [QX167].
+4. **First Time Donors by Month and Retention**: This report provides a monthly breakdown of first-time donors and their retention rates. By analyzing this data, you can identify trends in donor acquisition and retention over time, which is vital for understanding the lifetime value of different cohorts [QX74].
+5. **Cumulative Revenue per Cohort Member**: This metric tracks the total revenue generated by each cohort divided by the initial cohort size over multiple years. It provides a clear picture of the financial impact of each cohort, helping you assess their lifetime value [CI Hub Modified FINAL LARGE DOC (1), Page 30].
+By utilizing these analytics, you can gain a comprehensive understanding of the lifetime value of your donor cohorts. Remember to **blend these RFM-based analytics with engagement analytics for a better picture** of donor behavior and potential.</t>
+  </si>
+  <si>
+    <t>[QX102] | [QX13] | [QX10] | CI Hub Modified FINAL LARGE DOC (1) (Page 17) | seasonal giving patterns (Page 4)</t>
+  </si>
+  <si>
+    <t>To determine your peak giving month, you should focus on analyzing **Seasonal Giving Patterns**. This analysis will help you understand when donations are most frequently received throughout the year, revealing critical insights into donor behavior and timing for your fundraising efforts.
+1. **Seasonal Giving Patterns**: This analysis provides a detailed view of monthly and quarterly donation trends, allowing you to identify which month typically sees the highest volume of contributions. By examining these patterns, you can align your fundraising campaigns with periods of increased donor generosity, maximizing your outreach effectiveness [QX102].
+2. **Donor Gift Count Trends**: This analysis tracks the number of gifts received over time, which can help you identify fluctuations in giving frequency. By comparing gift counts across different months, you can pinpoint your peak giving periods and understand how they relate to overall donor engagement [QX10].
+3. **Segmentation Data from Last Fiscal Year-2**: Reviewing historical data on total annual giving can provide context for your current trends. By analyzing the giving behavior from two years ago, you can identify patterns that may still be relevant today, helping to forecast peak giving months based on past performance [QX102].
+4. **Cohort Analysis**: This involves grouping donors by shared characteristics or behaviors to reveal patterns in their giving. By examining cohorts over time, you can identify which segments of your donor base are most active during specific months, further clarifying your peak giving periods [QX102].
+5. **Retention Hub**: While this primarily focuses on donor retention, understanding when donors are most likely to give can also inform your retention strategies. If you know your peak giving month, you can tailor your stewardship efforts to ensure donors feel appreciated and engaged during that time [QX10].
+By leveraging these RFM-based analytics, you can gain a clearer picture of your peak giving month. However, to enhance your understanding, consider blending these RFM-based analytics with engagement analytics for a better picture. This will provide a more comprehensive view of donor behavior and preferences.</t>
+  </si>
+  <si>
+    <t>[QX7] | [QX50] | [QX73] | seasonal giving patterns (Page 2) | CI Hub Modified FINAL LARGE DOC (1) (Page 19)</t>
+  </si>
+  <si>
+    <t>To understand whether Giving Tuesday donors contribute at other times, you should focus on several key RFM-based analytics that can provide insights into donor behavior and patterns. Here are the specific analytics you should review:
+1. **Donor Retention Analysis**: This analysis will help you assess the retention rates of donors who contributed on Giving Tuesday compared to other periods. By examining how many of these donors return to give again, you can identify if they are likely to contribute outside of this specific event [QX50].
+2. **Seasonal Giving Patterns**: Review the seasonal trends in donor acquisition, particularly focusing on the months surrounding Giving Tuesday. This will help you identify if there are predictable giving habits among these donors, such as whether they tend to give again during the year-end holiday season or at other times [Seasonal Giving Patterns (Page 2)].
+3. **Cohort Analysis of New Donors**: Analyze the cohort of new donors acquired on Giving Tuesday to see if they exhibit different giving behaviors compared to those acquired at other times. This can help you understand their overall engagement and whether they are likely to become multi-year supporters [QX73].
+4. **First Gift Analysis**: Look at the total, average, median, and mode of first gifts from Giving Tuesday donors. This will provide insights into their giving patterns and help you tailor future outreach efforts to encourage additional contributions [QX73].
+5. **Re-engagement Strategies**: Consider developing a re-engagement sequence specifically for Giving Tuesday donors. This could involve personalized follow-ups that reference their past support, which may encourage them to give again at other times of the year [QX7].
+By focusing on these RFM-based analytics, you can gain a clearer picture of the giving behavior of your Giving Tuesday donors. However, to enhance your understanding, blend these RFM-based analytics with engagement analytics for a better picture. This will allow you to see how engagement efforts may influence their giving patterns.</t>
+  </si>
+  <si>
+    <t>[QX59] | [QX73] | [QX54] | seasonal giving patterns (Page 4) | CI Hub Modified FINAL LARGE DOC (1) (Page 18)</t>
+  </si>
+  <si>
+    <t>To identify which months produce the most new donors, you should focus on the following RFM-based analytics:
+1. **First-Time Donor Month Rankings (LFY)**: This analysis will help you track the number and value of first-time donors acquired each month over the last fiscal year. By reviewing this data, you can pinpoint specific months that consistently yield high acquisition rates for new donors, allowing you to replicate successful strategies in future campaigns [QX59].
+2. **First-Time Donors by Month (LFY)**: Similar to the previous metric, this analysis provides insights into the monthly trends of first-time donors. It can help you understand seasonal patterns and the effectiveness of your outreach efforts during different times of the year [QX73].
+3. **Seasonal Giving Patterns**: This analysis goes beyond just monthly donor counts; it provides a comprehensive view of how donor behavior changes throughout the year. By integrating seasonal insights into your fundraising plans, you can align your campaigns with the times when donors are most likely to give, thus maximizing your acquisition efforts [Seasonal Giving Patterns (Page 4)].
+4. **First-Time Donors Acquisition by Month**: This metric focuses on the acquisition of new donors and can help you identify trends and patterns in donor behavior over time. Understanding these patterns can inform your strategies for future donor acquisition [QX54].
+5. **Retention and Reactivation Campaigns**: While this is not directly about new donor acquisition, understanding the retention of new donors can provide insights into the effectiveness of your acquisition strategies. If you notice a drop in retention during certain months, it may indicate a need to adjust your acquisition tactics [Seasonal Giving Patterns (Page 4)].
+By analyzing these RFM-based metrics, you can gain a clearer picture of which months are most effective for acquiring new donors. Remember to blend these RFM-based analytics with engagement analytics for a better picture. This will allow you to tailor your outreach and stewardship efforts more effectively, ensuring that you capitalize on the months that yield the highest new donor acquisition.</t>
+  </si>
+  <si>
+    <t>[QX89] | [QX155] | [QX14] | CI Hub Modified FINAL LARGE DOC (1) (Page 21) | seasonal giving patterns (Page 4)</t>
+  </si>
+  <si>
+    <t>To identify which donors contributed significantly in a specific month, you should focus on the following RFM-based analytics:
+1. **Top Segment Gift Amount Trends (Annual) Analysis**: This analysis provides a historical overview of your top donor segment, allowing you to see which donors qualified as top contributors in the month of interest. By examining the total dollars contributed and the number of unique top donors, you can pinpoint who made significant contributions during that time [QX89].
+2. **Seasonal Giving Patterns**: This analysis will help you understand the monthly and quarterly donation patterns. By examining the seasonal peaks in giving, you can identify if the lift in donations during the specific month was due to many small contributions or a few large gifts. This insight can reveal vulnerabilities and opportunities in your fundraising strategy [seasonal giving patterns (Page 4)].
+3. **Average Gift Size Trends**: Reviewing the average gift sizes for the last three fiscal years can help you identify any increases in contributions from specific donors. This analysis highlights donors whose average gift size has increased, indicating potential opportunities for deeper engagement [QX155].
+4. **Retention Hub**: This analysis focuses on donor retention and can provide insights into which segments are most likely to return and contribute again. By understanding the percentage of donors who increased their gifts, you can identify those who may have contributed significantly in the month you are investigating [QX14].
+5. **Gift Size and Seasonality**: This analysis will help you assess whether the contributions in the specific month were driven by a few major donors or a broader base of smaller gifts. Understanding this composition can inform your future fundraising strategies and highlight key contributors [CI Hub Modified FINAL LARGE DOC (1) (Page 21)].
+By leveraging these RFM-based analytics, you can gain a clearer picture of donor behavior during the specific month in question. Remember to blend these RFM-based analytics with engagement analytics for a better picture.</t>
+  </si>
+  <si>
+    <t>[QX46] | [QX26] | [QX14] | PreventDonorAttrition (1) (Page 2) | CI Hub Modified FINAL LARGE DOC (1) (Page 44)</t>
+  </si>
+  <si>
+    <t>While the CI Hub does not directly predict future giving behavior, it provides valuable insights through RFM (Recency, Frequency, Monetary Value) metrics that can help you understand donor patterns and inform your strategies. Here are some analytics you should consider reviewing:
+1. **3-Year Consecutive Donor Retention Analysis**: This report will help you assess how well your organization retains donors over a three-year period. By understanding retention trends, you can identify which donor segments are more likely to continue giving and which may need re-engagement strategies [QX46].
+2. **First-Time Donor 13-Month Retention Analysis**: This analysis focuses on new donors and tracks their retention within the critical 13-month window after their first gift. It provides insights into how effectively you convert first-time donors into repeat supporters, which is crucial for long-term sustainability [QX26].
+3. **New Donor to Second Gift Conversion Analysis**: This report examines the behavior of new donors, specifically how many return to make a second gift. By segmenting these donors based on their initial gift size, you can identify patterns in retention and upgrading, which can inform your future fundraising strategies [QX14].
+4. **Predictive Analytics for At-Risk Donors**: While the CI Hub does not predict future behavior directly, it can help identify donors who may be at risk of attrition. By analyzing past giving patterns, you can proactively engage with these donors to encourage continued support [PreventDonorAttrition (1) (Page 2)].
+5. **Speed Curves and Donor Quality**: Understanding the speed at which donors make their second gift can reveal insights into donor quality and engagement. This analysis can help you refine your acquisition strategies and focus on nurturing high-potential donors [CI Hub Modified FINAL LARGE DOC (1) (Page 44)].
+To enhance your understanding of future giving behavior, consider blending these RFM-based analytics with engagement analytics for a better picture. This combination will provide a more comprehensive view of donor behavior and help you tailor your strategies effectively.</t>
+  </si>
+  <si>
+    <t>[QX140] | van Diepen 2009 Direct Marketing Charity RFM Segmentation (Page 26) | Shaker Nelson 2021 Grounded Theory Major Gift Relationships (Page 8) | Bhati McDonnell 2019 Online Giving Day Social Media One Pager (Page 10) | Meer Rosen 2009 ABCs Charitable Solicitation NBER WP15037 (Page 28) | Shaker 2018 Understanding Higher Education Fundraisers Report (Page 24)</t>
+  </si>
+  <si>
+    <t>To assess the reliability of your projection model, you should focus on several key RFM-based analytics that can provide insights into donor behavior and the effectiveness of your forecasting. Here are the specific analytics you should consider:
+1. **Forecasted vs. Actual Outcomes**: Compare your forecasted retained donors and projected revenue against the actual outcomes. This side-by-side analysis will help you identify discrepancies and understand where your model performs well or needs refinement. Tracking transition percentages (such as upgrade, downgrade, and lapse rates) will also provide insights into donor lifecycle behaviors [QX140].
+2. **Donor Segmentation Analysis**: Break down your performance by donor segments. This will allow you to see how different groups of donors are responding to your fundraising efforts and whether your model accurately predicts movements within these segments. Understanding the share of new and reengaged donors can also highlight areas where your model may need adjustments [QX140].
+3. **Retention Rates**: Analyze your donor retention rates over time. High retention rates can indicate that your projection model is reliable, while significant fluctuations may suggest that adjustments are necessary. This metric is crucial for understanding the effectiveness of your stewardship and acquisition efforts [QX140].
+4. **Transition Rates**: Look at the rates of donor transitions, including upgrades and downgrades. These metrics can provide insights into how well your model predicts donor behavior and can help you identify trends that may not be captured in your initial forecasts [QX140].
+5. **Value of New/Reengaged Donors**: Assess the rate and value of new and reengaged donors. This analysis can help you understand the effectiveness of your acquisition strategies and whether your model accurately reflects the potential revenue from these groups [QX140].
+By focusing on these RFM-based analytics, you can gain a clearer picture of the reliability of your projection model. Remember, blending these RFM-based analytics with engagement analytics will provide a better overall understanding of donor behavior and model accuracy.
+For further insights, consider reviewing industry reports and studies that discuss the importance of these metrics in forecasting and donor management [van Diepen 2009; Shaker Nelson 2021; Bhati McDonnell 2019; Meer Rosen 2009; Shaker 2018].</t>
+  </si>
+  <si>
+    <t>[QX153] | [QX159] | [QX155]</t>
+  </si>
+  <si>
+    <t>To understand how donors transition into major donors, it's essential to analyze their giving patterns and engagement levels through specific RFM (Recency, Frequency, Monetary Value) metrics. Here are some analytics you should focus on:
+1. **Donor Upgrade Pipeline**: This analysis identifies potential upgrade candidates from your top-segment donor pool. By examining donors who have consistently given at a stable level over the past two years, you can pinpoint those who may be ready to increase their contributions. This is crucial because it highlights individuals who have shown commitment and may be receptive to major gift solicitations [QX159].
+2. **Donors Whose Gift Size is Increasing**: Focus on donors with an 'I' score, indicating an increase in average gift size. These individuals are likely to be more receptive to further engagement or major gift solicitations. Recognizing and thanking these donors can enhance relationships and encourage them to consider larger contributions [QX153].
+3. **Retention Hub**: Tracking the retention rate of top donors over time is vital. By monitoring changes in average gift sizes and total donations from identified groups, you can assess the effectiveness of your engagement strategies. This will help you understand which donors are becoming more committed and may be on the path to becoming major donors [QX153].
+4. **Engagement Metrics**: While the CI Hub does not contain engagement data, it is important to blend RFM analytics with engagement analytics for a better picture. Metrics such as event attendance or participation in donor surveys can provide insights into how engaged these donors are, which is a critical factor in their journey toward becoming major donors [QX155].
+5. **Performance Scoring**: Utilize a four-character performance score based on historical giving data to assess each donor's contribution patterns. This score reflects not only their current contributions but also their giving trends over the past few years, helping you identify those who are likely to upgrade their giving levels [QX159].
+In summary, donors can be "made" into major donors through strategic engagement and recognition of their giving patterns. By focusing on the right RFM metrics and blending them with engagement analytics, you can effectively nurture these relationships and encourage higher levels of giving.</t>
+  </si>
+  <si>
+    <t>[QX161] | [QX16] | [QX68] | CI Hub Modified FINAL LARGE DOC (1) (Page 26)</t>
+  </si>
+  <si>
+    <t>To understand how long it typically takes to develop a major donor, you should focus on the **Average Tenure to Top Level Donor Analysis**. This analysis tracks the progression of donors from their first gift to the point they make a major gift, providing insights into the average time it takes for donors to reach this key giving threshold. By examining the timeline of each donor's contributions, you can identify patterns and benchmarks that inform your development strategies [QX16].
+Additionally, consider reviewing your **Donor Lifecycle Data**. This data will help you interpret the actual rates of donor progression within your organization, allowing you to compare your findings against sector benchmarks. For instance, healthy organizations often see a gradual retention decline rather than steep drop-offs, which can indicate successful long-term relationship building [CI Hub Modified FINAL LARGE DOC (1) (Page 26)].
+You may also want to analyze the **Retention Hub** to understand how effectively different donor segments are retained over time. This can help you identify which segments are more likely to become major donors and tailor your engagement strategies accordingly [QX161].
+Lastly, the **Donor Recapture Analytics** can provide insights into lapsed donors and their potential to return, which can be crucial for understanding the overall donor journey and improving your major donor development efforts [QX68].
+In summary, focus on the following analytics:
+1. Average Tenure to Top Level Donor Analysis
+2. Donor Lifecycle Data
+3. Retention Hub
+4. Donor Recapture Analytics
+These insights will help you develop a clearer picture of the time and strategies needed to cultivate major donors. Blend these RFM-based analytics with engagement analytics for a better picture.</t>
+  </si>
+  <si>
+    <t>[QX91] | [QX92] | [QX44] | CI Hub Modified FINAL LARGE DOC (1) (Page 6) | PreventDonorAttrition (1) (Page 2)</t>
+  </si>
+  <si>
+    <t>To understand what a successful major donor growth path looks like, you should focus on several key RFM (Recency, Frequency, Monetary Value) analytics that can provide insights into donor behavior and engagement. Here are the specific analytics you should consider:
+1. **Active Top Segment Analysis**: This involves tracking retention rates, average gift trends, and gift frequency for your highest-capacity donors. A decline in retention among this segment can significantly impact your revenue, so monitoring these metrics is crucial for understanding the health of your major donor base [QX44].
+2. **Top Donor Concentration**: Evaluate the cumulative percentage of revenue contributed by your top donors. This analysis will help you assess the effectiveness of your personalized outreach strategies and the overall engagement of your major donor segment [QX44].
+3. **Upgrade Opportunities**: Focus on measuring the movement of donors into higher giving brackets year over year. This will help you identify potential upgrade candidates and ensure that your segmentation reflects current donor behavior [QX92].
+4. **Donor Lifecycle Analysis**: Analyze the retention rates and upgrade patterns among your major donors. This will provide insights into how many of your donors are retained, renewed, or acquired each year, which is essential for understanding the dynamics of your major donor pipeline [QX44].
+5. **Year-Over-Year Retention Metrics**: Track the retention rates of your top 1,000 donors and monitor changes in total dollars raised from this group. This will help you evaluate the effectiveness of your engagement activities and the overall health of your major donor relationships [QX91].
+By focusing on these RFM-based analytics, you can gain a clearer picture of your major donor growth path. However, to enhance your understanding, consider blending these RFM-based analytics with engagement analytics for a better picture. This will allow you to assess how engagement strategies impact donor retention and upgrades, ultimately leading to a more robust major donor growth strategy.
+For further insights, you may want to refer to industry reports that discuss donor behavior trends and retention strategies, such as those from Blackbaud and other fundraising performance management communities [PreventDonorAttrition (1), Page 2].</t>
+  </si>
+  <si>
+    <t>[QX92] | [QX81] | [QX91] | CI Hub Modified FINAL LARGE DOC (1) (Page 6)</t>
+  </si>
+  <si>
+    <t>To reach the million-dollar lifetime giving mark, it's essential to focus on several key analytics that can help you understand donor behavior and optimize your fundraising strategies. Here are the specific analytics you should consider:
+1. **Active Top Segment Analysis**: This involves tracking retention rates, average gift trends, and gift frequency for your highest-capacity donors. A decline in retention within this segment can significantly impact your revenue, so it's crucial to monitor these metrics closely [QX92].
+2. **Donor Upgrade Pipeline**: Analyze the movement of donors into higher giving brackets. This includes monitoring upgrade patterns and retention rates within your middle segment, which often represents your best opportunity for upgrades. Understanding how many donors are progressing towards higher giving levels can help you strategize effectively [QX91].
+3. **Gift Size Distribution**: Review the distribution of gift sizes among your donors. This analysis can help you identify which segments are contributing most significantly to your fundraising efforts and where you might find opportunities for growth [QX92].
+4. **Retention Hub**: Focus on retention rates across all segments, particularly the top and middle segments. High retention rates in these groups are critical for achieving long-term giving goals, including reaching the million-dollar mark [QX81].
+5. **Small-Dollar Segment Analysis**: While individual gifts may be smaller, this segment can provide sustainability and future upgrade candidates. Monitoring participation trends and retention rates in this group can help ensure a steady flow of contributions over time [CI Hub Modified FINAL LARGE DOC (1) (Page 6)].
+By leveraging these RFM-based analytics, you can gain insights into donor behavior and tailor your outreach strategies accordingly. Remember, blending these RFM-based analytics with engagement analytics will provide a more comprehensive view of your donor relationships and help you reach your fundraising goals more effectively.</t>
+  </si>
+  <si>
+    <t>[QX167] | [QX159] | [QX158] | CI Hub Modified FINAL LARGE DOC (1) (Page 6)</t>
+  </si>
+  <si>
+    <t>To assess upgrade probabilities at each stage of your donor segments, you should focus on several key RFM-based analytics that can provide insights into donor behavior and potential for upgrades. Here are the specific analytics you should consider:
+1. **Top Segment Stable-Target Increase**: This analysis identifies upgrade candidates from your top-segment donor pool by examining donors who have consistently given at a stable level over the past two years. It utilizes historical giving data to assess contribution patterns, which can help you understand the likelihood of upgrades among your most loyal and high-capacity donors [QX159].
+2. **Bottom Segment Stable-Target Increase**: Similar to the top segment analysis, this analytic focuses on the bottom-segment donors who have shown stable giving patterns. By identifying those whose contributions have remained consistent or slightly increased, you can gauge the potential for upgrades within this segment [QX158]. 
+3. **Active Top Segment Analysis**: This analytic tracks retention rates, average gift trends, and gift frequency for your highest-capacity donors. Given that a decline in retention among this segment can significantly impact revenue, understanding these metrics will help you assess upgrade probabilities and the overall health of your top donor relationships [CI Hub Modified FINAL LARGE DOC (1) (Page 6)].
+4. **Active Middle Segment Analysis**: This analysis monitors upgrade patterns and retention rates within the middle segment, which often represents a strong upgrade pipeline. By focusing on this segment, you can identify potential candidates for upgrades and understand their giving behaviors [CI Hub Modified FINAL LARGE DOC (1) (Page 6)].
+5. **Donor Loyalty Analysis by Segment**: This analysis allows you to measure the success of your engagement strategies by establishing metrics such as increased donor retention rates and the number of donors transitioning to higher tiers. Regularly assessing these metrics will provide insights into the effectiveness of your strategies and the upgrade probabilities for each segment [QX167].
+By leveraging these RFM-based analytics, you can gain a clearer picture of upgrade probabilities at each stage of your donor segments. However, to enhance your understanding, consider blending these RFM-based analytics with engagement analytics for a better picture. This will allow you to incorporate factors such as donor interactions and engagement levels, which can further inform your upgrade strategies.</t>
+  </si>
+  <si>
+    <t>[QX44] | [QX17] | [QX81] | CI Hub Modified FINAL LARGE DOC (1) (Page 39)</t>
+  </si>
+  <si>
+    <t>To identify your most loyal long-term major donors, you should focus on several key RFM-based analytics that will provide insights into donor behavior and value. Here are the specific analyses you should consider:
+1. **Donor Lifecycle Analysis**: This analysis will help you understand the transitions of your donors, including retention rates among your major donor segment. By summarizing the total number of donors in each segment and their rates of upgrade, retention, downgrade, and lapse, you can pinpoint which major donors are consistently contributing and which may be at risk of attrition. This is crucial for targeting stewardship efforts effectively [QX17].
+2. **Top Donor Concentration**: Review the cumulative percentage of revenue contributed by your top 1,000 donors. This will allow you to track year-over-year retention and upgrade rates, providing a clear picture of who your most loyal donors are and how their contributions have evolved over time. This analysis is particularly valuable for assessing the impact of personalized engagement activities on donor loyalty [QX44].
+3. **Recency, Frequency, and Monetary Value (RFM) Metrics**: Analyze the recency of donations, frequency of giving, and the total monetary value contributed by your major donors. This will help you identify those who not only give regularly but also have a history of significant contributions. By focusing on these metrics, you can prioritize outreach to those who are most engaged and likely to continue their support [QX81].
+4. **Retention Hub**: Utilize this analysis to track the retention rates of your major donors over time. Understanding the patterns of donor retention can help you identify which donors are most loyal and how their giving behavior has changed. This can inform your strategies for maintaining and enhancing these relationships [QX44].
+5. **Segment Movement Analysis**: This analysis will allow you to evaluate the effectiveness of your donor engagement strategies by tracking how major donors move between segments (e.g., from Middle to High Value). By understanding these dynamics, you can tailor your communications and stewardship efforts to celebrate upgrades and address any potential downgrades [QX17].
+By focusing on these RFM-based analytics, you can gain a comprehensive understanding of your most loyal long-term major donors. Remember to blend these RFM-based analytics with engagement analytics for a better picture of donor loyalty and engagement.</t>
+  </si>
+  <si>
+    <t>[QX167] | [QX166] | [QX44] | CI Hub Modified FINAL LARGE DOC (1) (Page 6)</t>
+  </si>
+  <si>
+    <t>To predict which current donors may transition into major donors, you should focus on several key RFM (Recency, Frequency, Monetary Value) analytics that can provide insights into donor behavior and potential for increased giving. Here are the specific analytics you should consider:
+1. **Active Top Segment Analysis**: This analysis tracks retention rates, average gift trends, and gift frequency for your highest-capacity donors. A decline in retention within this segment can significantly impact revenue, making it crucial to monitor these metrics closely [CI Hub Modified FINAL LARGE DOC (1) (Page 6)].
+2. **Active Middle Segment Analysis**: This metric helps you monitor upgrade patterns and retention rates among your middle-tier donors. Since this segment often represents your best upgrade pipeline, understanding their giving behavior can help identify potential major donors [CI Hub Modified FINAL LARGE DOC (1) (Page 6)].
+3. **Donor Loyalty Analysis by Segment**: By analyzing the loyalty of donors across different segments, you can identify those who have a consistent giving history. Donors with a long streak of contributions, even if small, may be more likely to respond positively to targeted engagement efforts aimed at upgrading their giving [QX167].
+4. **Year-Over-Year Retention Metrics**: Tracking retention rates among your top donors over time can reveal trends that indicate which donors are likely to increase their contributions. This analysis can also help you assess the effectiveness of your engagement strategies [QX44].
+5. **Upgrade Pipeline Monitoring**: Evaluate the cumulative percentage of revenue contributed by your top donors and track changes in their giving patterns. This will help you identify which donors are moving towards major giving levels and allow you to tailor your outreach accordingly [QX166].
+By focusing on these RFM-based analytics, you can gain valuable insights into your current donor base and identify those who are most likely to become major donors. However, to enhance your predictions, consider blending these RFM-based analytics with engagement analytics for a better picture. This combination will provide a more comprehensive understanding of donor behavior and potential.</t>
+  </si>
+  <si>
+    <t>[QX178] | [QX173] | [QX11]</t>
+  </si>
+  <si>
+    <t>To create a comprehensive dashboard for your top donors, you should focus on several key analytics that will provide insights into their giving behavior and engagement. Here are the specific analytics you should consider:
+1. **Top Donor Analysis**: This analysis ranks your top 30 donors based on their total contributions from the last complete fiscal year. It will help you identify who your most significant supporters are and whether they are new, recaptured, or retained donors. This information is crucial for understanding donor loyalty and potential for future engagement [QX178].
+2. **Donor Segmentation**: Segment your donors into categories such as top, middle, and bottom based on their donation thresholds from the previous fiscal year. This will allow you to track year-to-date giving performance and compare it with the same period last year. Additionally, it evaluates changes in donor behavior, helping you tailor your engagement strategies effectively [QX173].
+3. **Lifetime Giving and Engagement Trends**: Analyze total lifetime giving, average annual giving over the last three fiscal years, and consecutive years of giving. This will provide a deeper understanding of each donor's commitment and help you identify those who may be ready for more targeted cultivation or those who need re-engagement [QX173].
+4. **Gift Count Trends**: Review the total number of gifts and total amount given per fiscal year over the last four years. This analysis will flag donors whose gift count in the last full fiscal year falls below their average for the preceding three years, indicating potential at-risk donors. This is essential for proactive engagement strategies [QX11].
+5. **Movement Categories**: Track shifts in donor engagement by categorizing donors into 'Increased', 'Decreased', 'Lapsed', and 'Recaptured'. This will help you identify which donors are increasing their giving and those who may need relationship repair or reassessment of your value proposition [QX173].
+By focusing on these analytics, you can create a dashboard that not only highlights your top donors but also provides actionable insights into their giving patterns and engagement levels. Remember to blend these RFM-based analytics with engagement analytics for a better picture.</t>
+  </si>
+  <si>
+    <t>[QX170] | [QX57] | [QX136] | CI Hub Modified FINAL LARGE DOC (1) (Page 19)</t>
+  </si>
+  <si>
+    <t>To assess how your top donors are tracking this year compared to last year, you should focus on several key RFM-based analytics that will provide insights into donor behavior and trends. Here are the specific analytics you should review:
+1. **Retention Rates**: Examine the retention rates of your top donors over the past year. This will help you understand how many of these donors have continued their support compared to the previous year. Tracking changes in retention rates can indicate the effectiveness of your engagement strategies and overall donor satisfaction [QX57].
+2. **Average Annual Giving**: Analyze the average annual giving of your top donors. This metric will show you whether their contributions have increased, decreased, or remained stable compared to last year. A rise in average giving can signal successful engagement and satisfaction, while a decline may require further investigation [QX170].
+3. **Donor Upgrade Pipeline**: Review the transition rates of your top donors to see if any have moved to higher giving tiers. This analysis can help you identify which donors are becoming more engaged and willing to increase their support, as well as those who may need additional cultivation to encourage upgrades [QX136].
+4. **Cumulative Value of Gifts**: Look at the cumulative value of gifts made by your top donors over the past year. This will help you quantify their overall impact and assess whether their giving patterns are consistent with previous years. Understanding the lifetime value of these donors can inform your future fundraising strategies [QX57].
+5. **Donor Retention by Acquisition Season**: If applicable, analyze how the retention rates of your top donors vary by the season in which they were acquired. This can provide insights into the effectiveness of your acquisition strategies and help you tailor your engagement efforts accordingly [CI Hub Modified FINAL LARGE DOC (1) (Page 19)].
+By focusing on these RFM-based analytics, you can gain a clearer picture of how your top donors are performing this year compared to last year. Remember to blend these RFM-based analytics with engagement analytics for a better picture, as engagement metrics can provide additional context to your findings.</t>
+  </si>
+  <si>
+    <t>[QX159] | [QX89] | [QX158] | CI Hub Modified FINAL LARGE DOC (1) (Page 14) | Nyman Pilbeam Baines Maklan 2016 Transformational Gifts Roles Accepted Manuscript (Page 16)</t>
+  </si>
+  <si>
+    <t>To identify the linchpin donors driving your current results, you should focus on several key RFM-based analytics that will help you understand donor behavior and contribution patterns. Here are the specific analytics you should consider:
+1. **Top Segment Stable-Target Increase**: This analytic identifies upgrade candidates from your top-segment donor pool by examining donors who have consistently given at a stable level over the past two years. It utilizes historical giving data to assess each donor's contribution patterns, focusing on those who have maintained or increased their giving. This will help you pinpoint the donors who are not only loyal but also have the potential to increase their contributions, thus driving your results [QX159].
+2. **Average and Median Gift Amounts**: By analyzing the average and median gift amounts from your top donors, you can determine whether your revenue trends are driven by a few large gifts or a broader base of support. This insight is crucial for understanding the impact of your linchpin donors and can guide your strategies for retention and upgrades [QX89].
+3. **Retention Hub**: This analytic focuses on donor retention rates, which can help you identify which donors are consistently contributing over time. Understanding retention patterns will allow you to recognize the linchpin donors who are vital to your fundraising success and may require tailored stewardship strategies to keep them engaged [QX158].
+4. **Donor Upgrade Pipeline**: This analysis can help you identify potential upgrade candidates within your donor base. By focusing on those who have shown consistent giving patterns, you can develop targeted strategies to encourage these donors to increase their contributions, thereby enhancing your overall fundraising results [QX159].
+5. **Concentration Patterns**: Reviewing the concentration of revenue from your top donors can provide insights into how reliant your organization is on these key contributors. For instance, if a significant portion of your revenue comes from a small percentage of donors, these individuals are likely your linchpins. Understanding this distribution can help you manage risk and identify opportunities for growth [CI Hub Modified FINAL LARGE DOC (1), Page 14].
+By leveraging these RFM-based analytics, you can gain a clearer picture of who your linchpin donors are and how they are influencing your current fundraising results. Remember to blend these RFM-based analytics with engagement analytics for a better picture.</t>
+  </si>
+  <si>
+    <t>[QX44] | [QX51] | [QX91] | CI Hub Modified FINAL LARGE DOC (1) (Page 48)</t>
+  </si>
+  <si>
+    <t>To analyze the characteristics and behaviors of your $1 million lifetime donors, you should focus on several key RFM-based analytics that can provide insights into their giving patterns and retention. Here are the specific analytics you should consider:
+1. **Donor Lifecycle Analysis**: This analysis will help you track the retention rates of your top donors, including those who have contributed $1 million or more over their lifetime. By examining how many of these donors are retained in the first, next three, or subsequent fiscal years, you can assess the effectiveness of your onboarding and stewardship strategies [QX51].
+2. **Top Donor Concentration**: Evaluate the cumulative percentage of revenue contributed by your top 1,000 donors, which includes your $1 million lifetime donors. This will allow you to monitor changes in their giving and retention over time, helping you understand the impact of personalized engagement activities on this critical segment [QX44].
+3. **Retention Hub**: Focus on year-over-year retention rates among your high-value donors. This will provide insights into how well you are maintaining relationships with your $1 million donors and whether your engagement strategies are effective in keeping them active and contributing [QX91].
+4. **Gift Amount Trends**: Analyze the trends in gift amounts from your top donors over time. This will help you identify patterns in their giving behavior, such as whether they are increasing their contributions, remaining stable, or declining, which can inform your future outreach and engagement strategies [QX91].
+5. **Second Gift Analytics**: This metric can help you understand how quickly your new donors, including those who may eventually reach the $1 million mark, develop ongoing relationships with your organization. Itâ€™s crucial to identify the early indicators of high lifetime value among new donors [CI Hub Modified FINAL LARGE DOC (1) (Page 48)].
+By focusing on these RFM-based analytics, you can gain a clearer picture of your $1 million lifetime donors and tailor your strategies to enhance their engagement and retention. Remember, blending these RFM-based analytics with engagement analytics will provide a better picture of their overall relationship with your organization.</t>
+  </si>
+  <si>
+    <t>Google Antigravity Update 5</t>
   </si>
 </sst>
 </file>
@@ -6593,9 +7355,9 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>'Benchmark Summary'!$A$6:$A$13</c:f>
+              <c:f>'Benchmark Summary'!$A$6:$A$14</c:f>
               <c:strCache>
-                <c:ptCount val="8"/>
+                <c:ptCount val="9"/>
                 <c:pt idx="0">
                   <c:v>Test 1</c:v>
                 </c:pt>
@@ -6620,15 +7382,18 @@
                 <c:pt idx="7">
                   <c:v>Google Antigravity Update 4</c:v>
                 </c:pt>
+                <c:pt idx="8">
+                  <c:v>Google Antigravity Update 5</c:v>
+                </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Benchmark Summary'!$B$6:$B$13</c:f>
+              <c:f>'Benchmark Summary'!$B$6:$B$14</c:f>
               <c:numCache>
                 <c:formatCode>0.0%</c:formatCode>
-                <c:ptCount val="8"/>
+                <c:ptCount val="9"/>
                 <c:pt idx="0">
                   <c:v>0.58409523809523822</c:v>
                 </c:pt>
@@ -6652,6 +7417,9 @@
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0.67255624999999997</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.63753906250000014</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7350,9 +8118,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>1589377</xdr:colOff>
+      <xdr:colOff>1593187</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>162560</xdr:rowOff>
+      <xdr:rowOff>158750</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -7394,15 +8162,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>653460</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>99680</xdr:rowOff>
+      <xdr:colOff>731399</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>103490</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>461517</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>24579</xdr:rowOff>
+      <xdr:colOff>541361</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>26484</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -7751,12 +8519,34 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="3">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{8DCDA536-11DA-4D6A-8F3D-202FA0D8FFB8}">
+  <we:reference id="wa200009404" version="1.0.0.8" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="wa200009404" version="1.0.0.8" store="en-US" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;c097ec8b-ff41-4bbc-bc6f-47ce6c0a98ef&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A94B463F-56DC-496D-A272-39FE0E1C5AFE}">
   <sheetPr>
     <tabColor indexed="44"/>
   </sheetPr>
-  <dimension ref="A2:E13"/>
+  <dimension ref="A2:E14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.42578125" bestFit="1" customWidth="1"/>
@@ -7935,9 +8725,1146 @@
         <v>935</v>
       </c>
     </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>1189</v>
+      </c>
+      <c r="B14" s="6">
+        <f>'Google Antigravity Update 5'!$H$1</f>
+        <v>0.63753906250000014</v>
+      </c>
+      <c r="C14">
+        <v>63</v>
+      </c>
+      <c r="D14">
+        <v>46125.686458333301</v>
+      </c>
+      <c r="E14" t="s">
+        <v>935</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{533CD98B-C0DE-45A4-9E79-CD064352CD6E}">
+  <dimension ref="A1:H65"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
+        <v>935</v>
+      </c>
+      <c r="H1" s="10">
+        <f>AVERAGE(C2:C65)</f>
+        <v>0.63753906250000014</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
+        <v>46125.68645833333</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="3">
+        <v>0.69699999999999995</v>
+      </c>
+      <c r="D2" t="s">
+        <v>1063</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
+        <v>46125.686666666668</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="3">
+        <v>0.68200000000000005</v>
+      </c>
+      <c r="D3" t="s">
+        <v>1065</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <v>46125.686886574076</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="3">
+        <v>0.60199999999999998</v>
+      </c>
+      <c r="D4" t="s">
+        <v>1067</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>1068</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
+        <v>46125.687106481484</v>
+      </c>
+      <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="3">
+        <v>0.68700000000000006</v>
+      </c>
+      <c r="D5" t="s">
+        <v>1069</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
+        <v>46125.687291666669</v>
+      </c>
+      <c r="B6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="3">
+        <v>0.624</v>
+      </c>
+      <c r="D6" t="s">
+        <v>1071</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>1072</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
+        <v>46125.687465277777</v>
+      </c>
+      <c r="B7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7" s="3">
+        <v>0.70399999999999996</v>
+      </c>
+      <c r="D7" t="s">
+        <v>1073</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>1074</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <v>46125.687673611108</v>
+      </c>
+      <c r="B8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="3">
+        <v>0.59199999999999997</v>
+      </c>
+      <c r="D8" t="s">
+        <v>1075</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A9" s="2">
+        <v>46125.687881944446</v>
+      </c>
+      <c r="B9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="3">
+        <v>0.66300000000000003</v>
+      </c>
+      <c r="D9" t="s">
+        <v>1077</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>1078</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A10" s="2">
+        <v>46125.688043981485</v>
+      </c>
+      <c r="B10" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" s="3">
+        <v>0.58399999999999996</v>
+      </c>
+      <c r="D10" t="s">
+        <v>1079</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>1080</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A11" s="2">
+        <v>46125.688252314816</v>
+      </c>
+      <c r="B11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C11" s="3">
+        <v>0.72299999999999998</v>
+      </c>
+      <c r="D11" t="s">
+        <v>1081</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>1082</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A12" s="2">
+        <v>46125.688437500001</v>
+      </c>
+      <c r="B12" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" s="3">
+        <v>0.432</v>
+      </c>
+      <c r="D12" t="s">
+        <v>1083</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>1084</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A13" s="2">
+        <v>46125.688564814816</v>
+      </c>
+      <c r="B13" t="s">
+        <v>39</v>
+      </c>
+      <c r="C13" s="3">
+        <v>0.69299999999999995</v>
+      </c>
+      <c r="D13" t="s">
+        <v>1085</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>1086</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A14" s="2">
+        <v>46125.688715277778</v>
+      </c>
+      <c r="B14" t="s">
+        <v>42</v>
+      </c>
+      <c r="C14" s="3">
+        <v>0.64900000000000002</v>
+      </c>
+      <c r="D14" t="s">
+        <v>1087</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>1088</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A15" s="2">
+        <v>46125.688900462963</v>
+      </c>
+      <c r="B15" t="s">
+        <v>44</v>
+      </c>
+      <c r="C15" s="3">
+        <v>0.63200000000000001</v>
+      </c>
+      <c r="D15" t="s">
+        <v>1089</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>1090</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A16" s="2">
+        <v>46125.689062500001</v>
+      </c>
+      <c r="B16" t="s">
+        <v>46</v>
+      </c>
+      <c r="C16" s="3">
+        <v>0.65100000000000002</v>
+      </c>
+      <c r="D16" t="s">
+        <v>1091</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>1092</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A17" s="2">
+        <v>46125.689259259256</v>
+      </c>
+      <c r="B17" t="s">
+        <v>49</v>
+      </c>
+      <c r="C17" s="3">
+        <v>0.64600000000000002</v>
+      </c>
+      <c r="D17" t="s">
+        <v>1093</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>1094</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A18" s="2">
+        <v>46125.689432870371</v>
+      </c>
+      <c r="B18" t="s">
+        <v>51</v>
+      </c>
+      <c r="C18" s="3">
+        <v>0.71299999999999997</v>
+      </c>
+      <c r="D18" t="s">
+        <v>1095</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>1096</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A19" s="2">
+        <v>46125.689606481479</v>
+      </c>
+      <c r="B19" t="s">
+        <v>54</v>
+      </c>
+      <c r="C19" s="3">
+        <v>0.68200000000000005</v>
+      </c>
+      <c r="D19" t="s">
+        <v>1097</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>1098</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A20" s="2">
+        <v>46125.689768518518</v>
+      </c>
+      <c r="B20" t="s">
+        <v>57</v>
+      </c>
+      <c r="C20" s="3">
+        <v>0.75700000000000001</v>
+      </c>
+      <c r="D20" t="s">
+        <v>1099</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>1100</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A21" s="2">
+        <v>46125.689976851849</v>
+      </c>
+      <c r="B21" t="s">
+        <v>60</v>
+      </c>
+      <c r="C21" s="3">
+        <v>0.45300000000000001</v>
+      </c>
+      <c r="D21" t="s">
+        <v>1101</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>1102</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A22" s="2">
+        <v>46125.690138888887</v>
+      </c>
+      <c r="B22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C22" s="3">
+        <v>0.625</v>
+      </c>
+      <c r="D22" t="s">
+        <v>1103</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>1104</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A23" s="2">
+        <v>46125.690324074072</v>
+      </c>
+      <c r="B23" t="s">
+        <v>66</v>
+      </c>
+      <c r="C23" s="3">
+        <v>0.63100000000000001</v>
+      </c>
+      <c r="D23" t="s">
+        <v>1105</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>1106</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A24" s="2">
+        <v>46125.690497685187</v>
+      </c>
+      <c r="B24" t="s">
+        <v>69</v>
+      </c>
+      <c r="C24" s="3">
+        <v>0.504</v>
+      </c>
+      <c r="D24" t="s">
+        <v>1107</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>1108</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A25" s="2">
+        <v>46125.690706018519</v>
+      </c>
+      <c r="B25" t="s">
+        <v>72</v>
+      </c>
+      <c r="C25" s="3">
+        <v>0.60499999999999998</v>
+      </c>
+      <c r="D25" t="s">
+        <v>1109</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>1110</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A26" s="2">
+        <v>46125.690844907411</v>
+      </c>
+      <c r="B26" t="s">
+        <v>74</v>
+      </c>
+      <c r="C26" s="3">
+        <v>0.59699999999999998</v>
+      </c>
+      <c r="D26" t="s">
+        <v>1111</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>1112</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A27" s="2">
+        <v>46125.691018518519</v>
+      </c>
+      <c r="B27" t="s">
+        <v>76</v>
+      </c>
+      <c r="C27" s="3">
+        <v>0.69599999999999995</v>
+      </c>
+      <c r="D27" t="s">
+        <v>1113</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>1114</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A28" s="2">
+        <v>46125.691180555557</v>
+      </c>
+      <c r="B28" t="s">
+        <v>79</v>
+      </c>
+      <c r="C28" s="3">
+        <v>0.71399999999999997</v>
+      </c>
+      <c r="D28" t="s">
+        <v>1115</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>1116</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A29" s="2">
+        <v>46125.691331018519</v>
+      </c>
+      <c r="B29" t="s">
+        <v>82</v>
+      </c>
+      <c r="C29" s="3">
+        <v>0.63600000000000001</v>
+      </c>
+      <c r="D29" t="s">
+        <v>1117</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>1118</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A30" s="2">
+        <v>46125.691504629627</v>
+      </c>
+      <c r="B30" t="s">
+        <v>85</v>
+      </c>
+      <c r="C30" s="3">
+        <v>0.61299999999999999</v>
+      </c>
+      <c r="D30" t="s">
+        <v>1119</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A31" s="2">
+        <v>46125.691666666666</v>
+      </c>
+      <c r="B31" t="s">
+        <v>88</v>
+      </c>
+      <c r="C31" s="3">
+        <v>0.62</v>
+      </c>
+      <c r="D31" t="s">
+        <v>1121</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>1122</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A32" s="2">
+        <v>46125.691817129627</v>
+      </c>
+      <c r="B32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C32" s="3">
+        <v>0.74199999999999999</v>
+      </c>
+      <c r="D32" t="s">
+        <v>1123</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>1124</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A33" s="2">
+        <v>46125.692002314812</v>
+      </c>
+      <c r="B33" t="s">
+        <v>94</v>
+      </c>
+      <c r="C33" s="3">
+        <v>0.60899999999999999</v>
+      </c>
+      <c r="D33" t="s">
+        <v>1125</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>1126</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A34" s="2">
+        <v>46125.692187499997</v>
+      </c>
+      <c r="B34" t="s">
+        <v>97</v>
+      </c>
+      <c r="C34" s="3">
+        <v>0.53200000000000003</v>
+      </c>
+      <c r="D34" t="s">
+        <v>1127</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>1128</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A35" s="2">
+        <v>46125.692384259259</v>
+      </c>
+      <c r="B35" t="s">
+        <v>100</v>
+      </c>
+      <c r="C35" s="3">
+        <v>0.66700000000000004</v>
+      </c>
+      <c r="D35" t="s">
+        <v>1129</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>1130</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A36" s="2">
+        <v>46125.69259259259</v>
+      </c>
+      <c r="B36" t="s">
+        <v>103</v>
+      </c>
+      <c r="C36" s="3">
+        <v>0.61399999999999999</v>
+      </c>
+      <c r="D36" t="s">
+        <v>1131</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>1132</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A37" s="2">
+        <v>46125.692754629628</v>
+      </c>
+      <c r="B37" t="s">
+        <v>106</v>
+      </c>
+      <c r="C37" s="3">
+        <v>0.53</v>
+      </c>
+      <c r="D37" t="s">
+        <v>1133</v>
+      </c>
+      <c r="E37" s="4" t="s">
+        <v>1134</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A38" s="2">
+        <v>46125.692916666667</v>
+      </c>
+      <c r="B38" t="s">
+        <v>109</v>
+      </c>
+      <c r="C38" s="3">
+        <v>0.71699999999999997</v>
+      </c>
+      <c r="D38" t="s">
+        <v>1135</v>
+      </c>
+      <c r="E38" s="4" t="s">
+        <v>1136</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A39" s="2">
+        <v>46125.693055555559</v>
+      </c>
+      <c r="B39" t="s">
+        <v>111</v>
+      </c>
+      <c r="C39" s="3">
+        <v>0.67200000000000004</v>
+      </c>
+      <c r="D39" t="s">
+        <v>1137</v>
+      </c>
+      <c r="E39" s="4" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A40" s="2">
+        <v>46125.69321759259</v>
+      </c>
+      <c r="B40" t="s">
+        <v>114</v>
+      </c>
+      <c r="C40" s="3">
+        <v>0.53700000000000003</v>
+      </c>
+      <c r="D40" t="s">
+        <v>1139</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A41" s="2">
+        <v>46125.693391203706</v>
+      </c>
+      <c r="B41" t="s">
+        <v>117</v>
+      </c>
+      <c r="C41" s="3">
+        <v>0.58899999999999997</v>
+      </c>
+      <c r="D41" t="s">
+        <v>1141</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>1142</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A42" s="2">
+        <v>46125.693576388891</v>
+      </c>
+      <c r="B42" t="s">
+        <v>120</v>
+      </c>
+      <c r="C42" s="3">
+        <v>0.46700000000000003</v>
+      </c>
+      <c r="D42" t="s">
+        <v>1143</v>
+      </c>
+      <c r="E42" s="4" t="s">
+        <v>1144</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A43" s="2">
+        <v>46125.693773148145</v>
+      </c>
+      <c r="B43" t="s">
+        <v>123</v>
+      </c>
+      <c r="C43" s="3">
+        <v>0.68899999999999995</v>
+      </c>
+      <c r="D43" t="s">
+        <v>1145</v>
+      </c>
+      <c r="E43" s="4" t="s">
+        <v>1146</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A44" s="2">
+        <v>46125.69394675926</v>
+      </c>
+      <c r="B44" t="s">
+        <v>126</v>
+      </c>
+      <c r="C44" s="3">
+        <v>0.48599999999999999</v>
+      </c>
+      <c r="D44" t="s">
+        <v>1147</v>
+      </c>
+      <c r="E44" s="4" t="s">
+        <v>1148</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A45" s="2">
+        <v>46125.694108796299</v>
+      </c>
+      <c r="B45" t="s">
+        <v>129</v>
+      </c>
+      <c r="C45" s="3">
+        <v>0.68600000000000005</v>
+      </c>
+      <c r="D45" t="s">
+        <v>1149</v>
+      </c>
+      <c r="E45" s="4" t="s">
+        <v>1150</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A46" s="2">
+        <v>46125.694293981483</v>
+      </c>
+      <c r="B46" t="s">
+        <v>132</v>
+      </c>
+      <c r="C46" s="3">
+        <v>0.65300000000000002</v>
+      </c>
+      <c r="D46" t="s">
+        <v>1151</v>
+      </c>
+      <c r="E46" s="4" t="s">
+        <v>1152</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A47" s="2">
+        <v>46125.694525462961</v>
+      </c>
+      <c r="B47" t="s">
+        <v>134</v>
+      </c>
+      <c r="C47" s="3">
+        <v>0.68300000000000005</v>
+      </c>
+      <c r="D47" t="s">
+        <v>1153</v>
+      </c>
+      <c r="E47" s="4" t="s">
+        <v>1154</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A48" s="2">
+        <v>46125.694687499999</v>
+      </c>
+      <c r="B48" t="s">
+        <v>137</v>
+      </c>
+      <c r="C48" s="3">
+        <v>0.504</v>
+      </c>
+      <c r="D48" t="s">
+        <v>1155</v>
+      </c>
+      <c r="E48" s="4" t="s">
+        <v>1156</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A49" s="2">
+        <v>46125.694872685184</v>
+      </c>
+      <c r="B49" t="s">
+        <v>140</v>
+      </c>
+      <c r="C49" s="3">
+        <v>0.67700000000000005</v>
+      </c>
+      <c r="D49" t="s">
+        <v>1157</v>
+      </c>
+      <c r="E49" s="4" t="s">
+        <v>1158</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A50" s="2">
+        <v>46125.695</v>
+      </c>
+      <c r="B50" t="s">
+        <v>142</v>
+      </c>
+      <c r="C50" s="3">
+        <v>0.63900000000000001</v>
+      </c>
+      <c r="D50" t="s">
+        <v>1159</v>
+      </c>
+      <c r="E50" s="4" t="s">
+        <v>1160</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A51" s="2">
+        <v>46125.695162037038</v>
+      </c>
+      <c r="B51" t="s">
+        <v>145</v>
+      </c>
+      <c r="C51" s="3">
+        <v>0.66300000000000003</v>
+      </c>
+      <c r="D51" t="s">
+        <v>1161</v>
+      </c>
+      <c r="E51" s="4" t="s">
+        <v>1162</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A52" s="2">
+        <v>46125.695416666669</v>
+      </c>
+      <c r="B52" t="s">
+        <v>148</v>
+      </c>
+      <c r="C52" s="3">
+        <v>0.627</v>
+      </c>
+      <c r="D52" t="s">
+        <v>1163</v>
+      </c>
+      <c r="E52" s="4" t="s">
+        <v>1164</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A53" s="2">
+        <v>46125.695590277777</v>
+      </c>
+      <c r="B53" t="s">
+        <v>151</v>
+      </c>
+      <c r="C53" s="3">
+        <v>0.36399999999999999</v>
+      </c>
+      <c r="D53" t="s">
+        <v>1165</v>
+      </c>
+      <c r="E53" s="4" t="s">
+        <v>1166</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A54" s="2">
+        <v>46125.695798611108</v>
+      </c>
+      <c r="B54" t="s">
+        <v>154</v>
+      </c>
+      <c r="C54" s="3">
+        <v>0.71199999999999997</v>
+      </c>
+      <c r="D54" t="s">
+        <v>1167</v>
+      </c>
+      <c r="E54" s="4" t="s">
+        <v>1168</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A55" s="2">
+        <v>46125.695949074077</v>
+      </c>
+      <c r="B55" t="s">
+        <v>157</v>
+      </c>
+      <c r="C55" s="3">
+        <v>0.69499999999999995</v>
+      </c>
+      <c r="D55" t="s">
+        <v>1169</v>
+      </c>
+      <c r="E55" s="4" t="s">
+        <v>1170</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A56" s="2">
+        <v>46125.696099537039</v>
+      </c>
+      <c r="B56" t="s">
+        <v>160</v>
+      </c>
+      <c r="C56" s="3">
+        <v>0.76300000000000001</v>
+      </c>
+      <c r="D56" t="s">
+        <v>1171</v>
+      </c>
+      <c r="E56" s="4" t="s">
+        <v>1172</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A57" s="2">
+        <v>46125.696273148147</v>
+      </c>
+      <c r="B57" t="s">
+        <v>163</v>
+      </c>
+      <c r="C57" s="3">
+        <v>0.74399999999999999</v>
+      </c>
+      <c r="D57" t="s">
+        <v>1173</v>
+      </c>
+      <c r="E57" s="4" t="s">
+        <v>1174</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A58" s="2">
+        <v>46125.696469907409</v>
+      </c>
+      <c r="B58" t="s">
+        <v>166</v>
+      </c>
+      <c r="C58" s="3">
+        <v>0.71199999999999997</v>
+      </c>
+      <c r="D58" t="s">
+        <v>1175</v>
+      </c>
+      <c r="E58" s="4" t="s">
+        <v>1176</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A59" s="2">
+        <v>46125.69667824074</v>
+      </c>
+      <c r="B59" t="s">
+        <v>168</v>
+      </c>
+      <c r="C59" s="3">
+        <v>0.68799999999999994</v>
+      </c>
+      <c r="D59" t="s">
+        <v>1177</v>
+      </c>
+      <c r="E59" s="4" t="s">
+        <v>1178</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A60" s="2">
+        <v>46125.696851851855</v>
+      </c>
+      <c r="B60" t="s">
+        <v>170</v>
+      </c>
+      <c r="C60" s="3">
+        <v>0.72899999999999998</v>
+      </c>
+      <c r="D60" t="s">
+        <v>1179</v>
+      </c>
+      <c r="E60" s="4" t="s">
+        <v>1180</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A61" s="2">
+        <v>46125.69703703704</v>
+      </c>
+      <c r="B61" t="s">
+        <v>173</v>
+      </c>
+      <c r="C61" s="3">
+        <v>0.71199999999999997</v>
+      </c>
+      <c r="D61" t="s">
+        <v>1181</v>
+      </c>
+      <c r="E61" s="4" t="s">
+        <v>1182</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A62" s="2">
+        <v>46125.697210648148</v>
+      </c>
+      <c r="B62" t="s">
+        <v>176</v>
+      </c>
+      <c r="C62" s="3">
+        <v>0.63600000000000001</v>
+      </c>
+      <c r="D62" t="s">
+        <v>1183</v>
+      </c>
+      <c r="E62" s="4" t="s">
+        <v>1184</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A63" s="2">
+        <v>46125.697372685187</v>
+      </c>
+      <c r="B63" t="s">
+        <v>178</v>
+      </c>
+      <c r="C63" s="3">
+        <v>0.61599999999999999</v>
+      </c>
+      <c r="D63" t="s">
+        <v>1185</v>
+      </c>
+      <c r="E63" s="4" t="s">
+        <v>1186</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A64" s="2">
+        <v>46125.697546296295</v>
+      </c>
+      <c r="B64" t="s">
+        <v>181</v>
+      </c>
+      <c r="C64" s="3">
+        <v>0.70399999999999996</v>
+      </c>
+      <c r="D64" t="s">
+        <v>1187</v>
+      </c>
+      <c r="E64" s="4" t="s">
+        <v>1188</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>792</v>
+      </c>
+      <c r="B65" t="s">
+        <v>793</v>
+      </c>
+      <c r="C65" s="3">
+        <v>0.63749999999999996</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -15749,6 +17676,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B446FD9-67AA-4836-A719-8C2263FFE390}">
   <dimension ref="A1:H65"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">

</xml_diff>